<commit_message>
Cập nhật trang web thẻ di động và bộ phân tích đa tầng mới nhất
</commit_message>
<xml_diff>
--- a/Kho_Can_Cu_Phap_Ly.xlsx
+++ b/Kho_Can_Cu_Phap_Ly.xlsx
@@ -1778,7 +1778,7 @@
       </c>
       <c r="J16" s="20" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Nghị định 24/2024/NĐ-CP</t>
+          <t>Bị thay thế bởi 24/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="K16" s="20" t="inlineStr">
@@ -5835,132 +5835,132 @@
       </c>
     </row>
     <row r="79" ht="26" customHeight="1">
-      <c r="A79" s="34" t="n">
+      <c r="A79" s="26" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="35" t="inlineStr">
+      <c r="B79" s="27" t="inlineStr">
         <is>
           <t>Xây dựng &amp; Quản lý dự án</t>
         </is>
       </c>
-      <c r="C79" s="36" t="inlineStr">
+      <c r="C79" s="28" t="inlineStr">
         <is>
           <t>Nghị định</t>
         </is>
       </c>
-      <c r="D79" s="37" t="inlineStr">
+      <c r="D79" s="29" t="inlineStr">
         <is>
           <t>05/2025/NĐ-CP</t>
         </is>
       </c>
-      <c r="E79" s="35" t="inlineStr">
+      <c r="E79" s="27" t="inlineStr">
         <is>
           <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
         </is>
       </c>
-      <c r="F79" s="38" t="inlineStr">
+      <c r="F79" s="30" t="inlineStr">
         <is>
           <t>Chính phủ</t>
         </is>
       </c>
-      <c r="G79" s="36" t="inlineStr">
+      <c r="G79" s="28" t="inlineStr">
         <is>
           <t>06/01/2025</t>
         </is>
       </c>
-      <c r="H79" s="36" t="inlineStr">
+      <c r="H79" s="28" t="inlineStr">
         <is>
           <t>06/01/2025</t>
         </is>
       </c>
-      <c r="I79" s="34" t="inlineStr">
+      <c r="I79" s="31" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
       </c>
-      <c r="J79" s="35" t="inlineStr">
+      <c r="J79" s="27" t="inlineStr">
         <is>
           <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP; được sửa đổi bởi Nghị định 48/2026/NĐ-CP</t>
         </is>
       </c>
-      <c r="K79" s="35" t="inlineStr">
+      <c r="K79" s="27" t="inlineStr">
         <is>
           <t>Quy định phân quyền và cắt giảm thủ tục cấp Giấy phép môi trường, Đăng ký môi trường</t>
         </is>
       </c>
-      <c r="L79" s="35" t="inlineStr">
+      <c r="L79" s="27" t="inlineStr">
         <is>
           <t>MOI_TRUONG, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M79" s="39" t="inlineStr"/>
-      <c r="N79" s="36" t="inlineStr">
+      <c r="M79" s="32" t="inlineStr"/>
+      <c r="N79" s="28" t="inlineStr">
         <is>
           <t>2026-08-21 11:07</t>
         </is>
       </c>
     </row>
     <row r="80" ht="26" customHeight="1">
-      <c r="A80" s="34" t="n">
+      <c r="A80" s="19" t="n">
         <v>79</v>
       </c>
-      <c r="B80" s="35" t="inlineStr">
+      <c r="B80" s="20" t="inlineStr">
         <is>
           <t>Xây dựng &amp; Quản lý dự án</t>
         </is>
       </c>
-      <c r="C80" s="36" t="inlineStr">
+      <c r="C80" s="21" t="inlineStr">
         <is>
           <t>Nghị định</t>
         </is>
       </c>
-      <c r="D80" s="37" t="inlineStr">
+      <c r="D80" s="22" t="inlineStr">
         <is>
           <t>48/2026/NĐ-CP</t>
         </is>
       </c>
-      <c r="E80" s="35" t="inlineStr">
+      <c r="E80" s="20" t="inlineStr">
         <is>
           <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP ngày 06 tháng 01 năm 2025</t>
         </is>
       </c>
-      <c r="F80" s="38" t="inlineStr">
+      <c r="F80" s="23" t="inlineStr">
         <is>
           <t>Chính phủ</t>
         </is>
       </c>
-      <c r="G80" s="36" t="inlineStr">
+      <c r="G80" s="21" t="inlineStr">
         <is>
           <t>15/05/2026</t>
         </is>
       </c>
-      <c r="H80" s="36" t="inlineStr">
+      <c r="H80" s="21" t="inlineStr">
         <is>
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="I80" s="34" t="inlineStr">
+      <c r="I80" s="31" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
       </c>
-      <c r="J80" s="35" t="inlineStr">
+      <c r="J80" s="20" t="inlineStr">
         <is>
           <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP và Nghị định số 05/2025/NĐ-CP</t>
         </is>
       </c>
-      <c r="K80" s="35" t="inlineStr">
+      <c r="K80" s="20" t="inlineStr">
         <is>
           <t>Đơn giản hóa tối đa thủ tục môi trường cho các công trình xây dựng và dự án đầu tư công hiện hành</t>
         </is>
       </c>
-      <c r="L80" s="35" t="inlineStr">
+      <c r="L80" s="20" t="inlineStr">
         <is>
           <t>ALL, MOI_TRUONG, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M80" s="39" t="inlineStr"/>
-      <c r="N80" s="36" t="inlineStr">
+      <c r="M80" s="25" t="inlineStr"/>
+      <c r="N80" s="21" t="inlineStr">
         <is>
           <t>2026-08-21 11:07</t>
         </is>

</xml_diff>

<commit_message>
Cập nhật chuỗi mắt xích pháp lý chuẩn xác: 30/2009/QH12 hết hiệu lực và thay thế bởi 47/2024/QH15
</commit_message>
<xml_diff>
--- a/Kho_Can_Cu_Phap_Ly.xlsx
+++ b/Kho_Can_Cu_Phap_Ly.xlsx
@@ -45,13 +45,13 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00991B1B"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00991B1B"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -76,8 +76,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
-        <bgColor rgb="00D1FAE5"/>
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -88,8 +88,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
-        <bgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -174,11 +174,11 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -657,7 +657,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Luật Quy hoạch đô thị năm 2009 (sửa đổi, bổ sung bởi Luật số 35/2018/QH14)</t>
+          <t>Luật Quy hoạch đô thị năm 2009</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -677,12 +677,12 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>Đang có hiệu lực</t>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Bị thay thế bởi Luật Quy hoạch đô thị và nông thôn số 47/2024/QH15</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -698,7 +698,7 @@
       <c r="M2" s="8" t="inlineStr"/>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
           <t>30/06/2015</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -761,10 +761,10 @@
           <t>ALL, QUY_HOACH, TV-01, TV-02, QLDA</t>
         </is>
       </c>
-      <c r="M3" s="14" t="inlineStr"/>
+      <c r="M3" s="15" t="inlineStr"/>
       <c r="N3" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
           <t>01/01/2023</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -830,7 +830,7 @@
       <c r="M4" s="8" t="inlineStr"/>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
           <t>15/02/2020</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -893,10 +893,10 @@
           <t>QUY_HOACH, CHI_PHI_QUY_HOACH, DU_TOAN, TV-01</t>
         </is>
       </c>
-      <c r="M5" s="14" t="inlineStr"/>
+      <c r="M5" s="15" t="inlineStr"/>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
           <t>05/07/2021</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -962,7 +962,7 @@
       <c r="M6" s="8" t="inlineStr"/>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
           <t>01/01/2019</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -1025,10 +1025,10 @@
           <t>KHAO_SAT, DO_DAC, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M7" s="14" t="inlineStr"/>
+      <c r="M7" s="15" t="inlineStr"/>
       <c r="N7" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
           <t>01/05/2019</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -1094,7 +1094,7 @@
       <c r="M8" s="8" t="inlineStr"/>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
           <t>01/01/2015</t>
         </is>
       </c>
-      <c r="I9" s="15" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -1157,10 +1157,10 @@
           <t>ALL, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M9" s="14" t="inlineStr"/>
+      <c r="M9" s="15" t="inlineStr"/>
       <c r="N9" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I10" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -1226,7 +1226,7 @@
       <c r="M10" s="8" t="inlineStr"/>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
           <t>01/01/2021</t>
         </is>
       </c>
-      <c r="I11" s="15" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -1289,10 +1289,10 @@
           <t>ALL, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M11" s="14" t="inlineStr"/>
+      <c r="M11" s="15" t="inlineStr"/>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
           <t>03/03/2021</t>
         </is>
       </c>
-      <c r="I12" s="15" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -1358,7 +1358,7 @@
       <c r="M12" s="8" t="inlineStr"/>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
           <t>15/02/2025</t>
         </is>
       </c>
-      <c r="I13" s="15" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -1421,10 +1421,10 @@
           <t>ALL, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M13" s="14" t="inlineStr"/>
+      <c r="M13" s="15" t="inlineStr"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -1490,7 +1490,7 @@
       <c r="M14" s="8" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
           <t>20/06/2023</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -1553,10 +1553,10 @@
           <t>ALL, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M15" s="14" t="inlineStr"/>
+      <c r="M15" s="15" t="inlineStr"/>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
           <t>28/02/2027</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I16" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -1622,7 +1622,7 @@
       <c r="M16" s="8" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
           <t>01/01/2024</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -1685,10 +1685,10 @@
           <t>ALL, DAU_THAU, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M17" s="14" t="inlineStr"/>
+      <c r="M17" s="15" t="inlineStr"/>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
           <t>15/01/2025</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="I18" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -1754,7 +1754,7 @@
       <c r="M18" s="8" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
           <t>01/08/2025</t>
         </is>
       </c>
-      <c r="I19" s="15" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -1817,10 +1817,10 @@
           <t>ALL, DAU_THAU, KHLCNT</t>
         </is>
       </c>
-      <c r="M19" s="14" t="inlineStr"/>
+      <c r="M19" s="15" t="inlineStr"/>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
           <t>01/07/2014</t>
         </is>
       </c>
-      <c r="I20" s="15" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -1886,7 +1886,7 @@
       <c r="M20" s="8" t="inlineStr"/>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
           <t>27/02/2024</t>
         </is>
       </c>
-      <c r="I21" s="15" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -1949,10 +1949,10 @@
           <t>ALL, DAU_THAU, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M21" s="14" t="inlineStr"/>
+      <c r="M21" s="15" t="inlineStr"/>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I22" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -2018,7 +2018,7 @@
       <c r="M22" s="8" t="inlineStr"/>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
           <t>15/08/2014</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -2081,10 +2081,10 @@
           <t>DAU_THAU, LICHSU</t>
         </is>
       </c>
-      <c r="M23" s="14" t="inlineStr"/>
+      <c r="M23" s="15" t="inlineStr"/>
       <c r="N23" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
           <t>26/04/2024</t>
         </is>
       </c>
-      <c r="I24" s="15" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -2150,7 +2150,7 @@
       <c r="M24" s="8" t="inlineStr"/>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2193,7 @@
           <t>01/01/2025</t>
         </is>
       </c>
-      <c r="I25" s="15" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -2213,10 +2213,10 @@
           <t>ALL, DAU_THAU, E_HSMT, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, XD-01</t>
         </is>
       </c>
-      <c r="M25" s="14" t="inlineStr"/>
+      <c r="M25" s="15" t="inlineStr"/>
       <c r="N25" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="I26" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -2282,7 +2282,7 @@
       <c r="M26" s="8" t="inlineStr"/>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
           <t>15/06/2024</t>
         </is>
       </c>
-      <c r="I27" s="15" t="inlineStr">
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -2345,10 +2345,10 @@
           <t>ALL, DAU_THAU, E_HSMT, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, XD-01</t>
         </is>
       </c>
-      <c r="M27" s="14" t="inlineStr"/>
+      <c r="M27" s="15" t="inlineStr"/>
       <c r="N27" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
           <t>01/01/2025</t>
         </is>
       </c>
-      <c r="I28" s="15" t="inlineStr">
+      <c r="I28" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -2414,7 +2414,7 @@
       <c r="M28" s="8" t="inlineStr"/>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="I29" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -2477,10 +2477,10 @@
           <t>ALL, DAU_THAU, E_HSMT, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, XD-01</t>
         </is>
       </c>
-      <c r="M29" s="14" t="inlineStr"/>
+      <c r="M29" s="15" t="inlineStr"/>
       <c r="N29" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2523,7 @@
           <t>30/09/2024</t>
         </is>
       </c>
-      <c r="I30" s="15" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -2546,7 +2546,7 @@
       <c r="M30" s="8" t="inlineStr"/>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
+      <c r="I31" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -2609,10 +2609,10 @@
           <t>DAU_THAU, DAU_TU_KINH_DOANH, PPP</t>
         </is>
       </c>
-      <c r="M31" s="14" t="inlineStr"/>
+      <c r="M31" s="15" t="inlineStr"/>
       <c r="N31" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2655,7 @@
           <t>09/02/2021</t>
         </is>
       </c>
-      <c r="I32" s="15" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -2678,7 +2678,7 @@
       <c r="M32" s="8" t="inlineStr"/>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="I33" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -2741,10 +2741,10 @@
           <t>ALL, DU_TOAN, QUAN_LY_CHI_PHI, TV-01, TV-02, TV-03, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M33" s="14" t="inlineStr"/>
+      <c r="M33" s="15" t="inlineStr"/>
       <c r="N33" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
           <t>15/10/2021</t>
         </is>
       </c>
-      <c r="I34" s="7" t="inlineStr">
+      <c r="I34" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -2810,7 +2810,7 @@
       <c r="M34" s="8" t="inlineStr"/>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
           <t>15/10/2021</t>
         </is>
       </c>
-      <c r="I35" s="15" t="inlineStr">
+      <c r="I35" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -2873,10 +2873,10 @@
           <t>ALL, DINH_MUC, DU_TOAN, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-08, TV-09, XD-01</t>
         </is>
       </c>
-      <c r="M35" s="14" t="inlineStr"/>
+      <c r="M35" s="15" t="inlineStr"/>
       <c r="N35" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2919,7 @@
           <t>15/10/2021</t>
         </is>
       </c>
-      <c r="I36" s="7" t="inlineStr">
+      <c r="I36" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -2942,7 +2942,7 @@
       <c r="M36" s="8" t="inlineStr"/>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2985,7 @@
           <t>15/02/2024</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="I37" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3005,10 +3005,10 @@
           <t>ALL, DU_TOAN, QUAN_LY_CHI_PHI, TV-01, TV-02, TV-03, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M37" s="14" t="inlineStr"/>
+      <c r="M37" s="15" t="inlineStr"/>
       <c r="N37" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
           <t>01/03/2025</t>
         </is>
       </c>
-      <c r="I38" s="7" t="inlineStr">
+      <c r="I38" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3074,7 +3074,7 @@
       <c r="M38" s="8" t="inlineStr"/>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
           <t>15/10/2024</t>
         </is>
       </c>
-      <c r="I39" s="15" t="inlineStr">
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -3137,10 +3137,10 @@
           <t>ALL, DINH_MUC, DU_TOAN, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-08, TV-09, XD-01</t>
         </is>
       </c>
-      <c r="M39" s="14" t="inlineStr"/>
+      <c r="M39" s="15" t="inlineStr"/>
       <c r="N39" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
           <t>01/08/2026</t>
         </is>
       </c>
-      <c r="I40" s="7" t="inlineStr">
+      <c r="I40" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3206,7 +3206,7 @@
       <c r="M40" s="8" t="inlineStr"/>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3249,7 @@
           <t>19/05/2023</t>
         </is>
       </c>
-      <c r="I41" s="15" t="inlineStr">
+      <c r="I41" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -3269,10 +3269,10 @@
           <t>SUAT_VON_DAU_TU, TMDT, TV-01, TV-02, TV-03, TV-04</t>
         </is>
       </c>
-      <c r="M41" s="14" t="inlineStr"/>
+      <c r="M41" s="15" t="inlineStr"/>
       <c r="N41" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
           <t>25/04/2025</t>
         </is>
       </c>
-      <c r="I42" s="15" t="inlineStr">
+      <c r="I42" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -3338,7 +3338,7 @@
       <c r="M42" s="8" t="inlineStr"/>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
           <t>26/01/2021</t>
         </is>
       </c>
-      <c r="I43" s="7" t="inlineStr">
+      <c r="I43" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3401,10 +3401,10 @@
           <t>CHAT_LUONG, NGHIEM_THU, TV-01, TV-02, TV-04, TV-05, TV-07, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M43" s="14" t="inlineStr"/>
+      <c r="M43" s="15" t="inlineStr"/>
       <c r="N43" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3447,7 +3447,7 @@
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="I44" s="7" t="inlineStr">
+      <c r="I44" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3470,7 +3470,7 @@
       <c r="M44" s="8" t="inlineStr"/>
       <c r="N44" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3513,7 @@
           <t>15/10/2021</t>
         </is>
       </c>
-      <c r="I45" s="7" t="inlineStr">
+      <c r="I45" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3533,10 +3533,10 @@
           <t>CHAT_LUONG, NGHIEM_THU, TV-01, TV-02, TV-04, TV-05, TV-07, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M45" s="14" t="inlineStr"/>
+      <c r="M45" s="15" t="inlineStr"/>
       <c r="N45" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
           <t>01/08/2026</t>
         </is>
       </c>
-      <c r="I46" s="7" t="inlineStr">
+      <c r="I46" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3602,7 +3602,7 @@
       <c r="M46" s="8" t="inlineStr"/>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
           <t>01/12/2023</t>
         </is>
       </c>
-      <c r="I47" s="7" t="inlineStr">
+      <c r="I47" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3665,10 +3665,10 @@
           <t>PCCC, THIET_KE, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M47" s="14" t="inlineStr"/>
+      <c r="M47" s="15" t="inlineStr"/>
       <c r="N47" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
           <t>10/01/2021</t>
         </is>
       </c>
-      <c r="I48" s="15" t="inlineStr">
+      <c r="I48" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -3734,7 +3734,7 @@
       <c r="M48" s="8" t="inlineStr"/>
       <c r="N48" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3777,7 @@
           <t>01/07/2025</t>
         </is>
       </c>
-      <c r="I49" s="7" t="inlineStr">
+      <c r="I49" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3797,10 +3797,10 @@
           <t>ALL, PCCC, THIET_KE, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M49" s="14" t="inlineStr"/>
+      <c r="M49" s="15" t="inlineStr"/>
       <c r="N49" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3843,7 @@
           <t>15/05/2024</t>
         </is>
       </c>
-      <c r="I50" s="15" t="inlineStr">
+      <c r="I50" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -3866,7 +3866,7 @@
       <c r="M50" s="8" t="inlineStr"/>
       <c r="N50" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3909,7 @@
           <t>01/04/2021</t>
         </is>
       </c>
-      <c r="I51" s="15" t="inlineStr">
+      <c r="I51" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -3929,10 +3929,10 @@
           <t>HOP_DONG, XD-01, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01</t>
         </is>
       </c>
-      <c r="M51" s="14" t="inlineStr"/>
+      <c r="M51" s="15" t="inlineStr"/>
       <c r="N51" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3975,7 @@
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="I52" s="7" t="inlineStr">
+      <c r="I52" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -3998,7 +3998,7 @@
       <c r="M52" s="8" t="inlineStr"/>
       <c r="N52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
           <t>20/04/2023</t>
         </is>
       </c>
-      <c r="I53" s="7" t="inlineStr">
+      <c r="I53" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4061,10 +4061,10 @@
           <t>HOP_DONG, XD-01, TV-04, TV-08</t>
         </is>
       </c>
-      <c r="M53" s="14" t="inlineStr"/>
+      <c r="M53" s="15" t="inlineStr"/>
       <c r="N53" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4107,7 @@
           <t>28/12/2012</t>
         </is>
       </c>
-      <c r="I54" s="7" t="inlineStr">
+      <c r="I54" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4130,7 +4130,7 @@
       <c r="M54" s="8" t="inlineStr"/>
       <c r="N54" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4173,7 +4173,7 @@
           <t>01/01/2023</t>
         </is>
       </c>
-      <c r="I55" s="7" t="inlineStr">
+      <c r="I55" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4193,10 +4193,10 @@
           <t>PTV-01, BAO_HIEM</t>
         </is>
       </c>
-      <c r="M55" s="14" t="inlineStr"/>
+      <c r="M55" s="15" t="inlineStr"/>
       <c r="N55" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4239,7 +4239,7 @@
           <t>06/09/2023</t>
         </is>
       </c>
-      <c r="I56" s="7" t="inlineStr">
+      <c r="I56" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4262,7 +4262,7 @@
       <c r="M56" s="8" t="inlineStr"/>
       <c r="N56" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4305,7 +4305,7 @@
           <t>01/08/2026</t>
         </is>
       </c>
-      <c r="I57" s="7" t="inlineStr">
+      <c r="I57" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4325,10 +4325,10 @@
           <t>ALL, PTV-01, BAO_HIEM, XD-01</t>
         </is>
       </c>
-      <c r="M57" s="14" t="inlineStr"/>
+      <c r="M57" s="15" t="inlineStr"/>
       <c r="N57" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
           <t>10/02/2016</t>
         </is>
       </c>
-      <c r="I58" s="15" t="inlineStr">
+      <c r="I58" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -4394,7 +4394,7 @@
       <c r="M58" s="8" t="inlineStr"/>
       <c r="N58" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4437,7 @@
           <t>01/01/2012</t>
         </is>
       </c>
-      <c r="I59" s="7" t="inlineStr">
+      <c r="I59" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4457,10 +4457,10 @@
           <t>TV-09, KIEM_TOAN</t>
         </is>
       </c>
-      <c r="M59" s="14" t="inlineStr"/>
+      <c r="M59" s="15" t="inlineStr"/>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4503,7 @@
           <t>01/01/2016</t>
         </is>
       </c>
-      <c r="I60" s="7" t="inlineStr">
+      <c r="I60" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4526,7 +4526,7 @@
       <c r="M60" s="8" t="inlineStr"/>
       <c r="N60" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4569,7 +4569,7 @@
           <t>01/01/2025</t>
         </is>
       </c>
-      <c r="I61" s="7" t="inlineStr">
+      <c r="I61" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4589,10 +4589,10 @@
           <t>ALL, DAU_TU_CONG, CHU_TRUONG, TV-01, TV-02, TV-03, TV-09</t>
         </is>
       </c>
-      <c r="M61" s="14" t="inlineStr"/>
+      <c r="M61" s="15" t="inlineStr"/>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4635,7 +4635,7 @@
           <t>01/01/2020</t>
         </is>
       </c>
-      <c r="I62" s="15" t="inlineStr">
+      <c r="I62" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -4658,7 +4658,7 @@
       <c r="M62" s="8" t="inlineStr"/>
       <c r="N62" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
           <t>01/01/2022</t>
         </is>
       </c>
-      <c r="I63" s="15" t="inlineStr">
+      <c r="I63" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -4721,10 +4721,10 @@
           <t>ALL, QUYET_TOAN, TAI_CHINH, TV-09, XD-01</t>
         </is>
       </c>
-      <c r="M63" s="14" t="inlineStr"/>
+      <c r="M63" s="15" t="inlineStr"/>
       <c r="N63" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4767,7 +4767,7 @@
           <t>01/01/2025</t>
         </is>
       </c>
-      <c r="I64" s="7" t="inlineStr">
+      <c r="I64" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4790,7 +4790,7 @@
       <c r="M64" s="8" t="inlineStr"/>
       <c r="N64" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4833,7 @@
           <t>26/11/2018</t>
         </is>
       </c>
-      <c r="I65" s="7" t="inlineStr">
+      <c r="I65" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4853,10 +4853,10 @@
           <t>BQP, DOANH_TRAI, TV-01, TV-02, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M65" s="14" t="inlineStr"/>
+      <c r="M65" s="15" t="inlineStr"/>
       <c r="N65" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4899,7 +4899,7 @@
           <t>20/11/2021</t>
         </is>
       </c>
-      <c r="I66" s="15" t="inlineStr">
+      <c r="I66" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -4922,7 +4922,7 @@
       <c r="M66" s="8" t="inlineStr"/>
       <c r="N66" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
           <t>12/02/2022</t>
         </is>
       </c>
-      <c r="I67" s="7" t="inlineStr">
+      <c r="I67" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -4985,10 +4985,10 @@
           <t>CHAT_LUONG, NGHIEM_THU, TV-01, TV-02, TV-04, TV-05, TV-07, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M67" s="14" t="inlineStr"/>
+      <c r="M67" s="15" t="inlineStr"/>
       <c r="N67" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5031,7 @@
           <t>26/12/2024</t>
         </is>
       </c>
-      <c r="I68" s="7" t="inlineStr">
+      <c r="I68" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5054,7 +5054,7 @@
       <c r="M68" s="8" t="inlineStr"/>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
           <t>20/11/2023</t>
         </is>
       </c>
-      <c r="I69" s="15" t="inlineStr">
+      <c r="I69" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -5117,10 +5117,10 @@
           <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M69" s="14" t="inlineStr"/>
+      <c r="M69" s="15" t="inlineStr"/>
       <c r="N69" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5163,7 @@
           <t>10/02/2025</t>
         </is>
       </c>
-      <c r="I70" s="15" t="inlineStr">
+      <c r="I70" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -5186,7 +5186,7 @@
       <c r="M70" s="8" t="inlineStr"/>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
           <t>20/06/2025</t>
         </is>
       </c>
-      <c r="I71" s="7" t="inlineStr">
+      <c r="I71" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5249,10 +5249,10 @@
           <t>CHAT_LUONG, NGHIEM_THU, TV-01, TV-02, TV-04, TV-05, TV-07, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M71" s="14" t="inlineStr"/>
+      <c r="M71" s="15" t="inlineStr"/>
       <c r="N71" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5295,7 +5295,7 @@
           <t>09/07/2026</t>
         </is>
       </c>
-      <c r="I72" s="7" t="inlineStr">
+      <c r="I72" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5318,7 +5318,7 @@
       <c r="M72" s="8" t="inlineStr"/>
       <c r="N72" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
           <t>30/08/2026</t>
         </is>
       </c>
-      <c r="I73" s="7" t="inlineStr">
+      <c r="I73" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5381,10 +5381,10 @@
           <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M73" s="14" t="inlineStr"/>
+      <c r="M73" s="15" t="inlineStr"/>
       <c r="N73" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
           <t>11/03/2025</t>
         </is>
       </c>
-      <c r="I74" s="7" t="inlineStr">
+      <c r="I74" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5450,7 +5450,7 @@
       <c r="M74" s="8" t="inlineStr"/>
       <c r="N74" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5493,7 @@
           <t>01/01/2018</t>
         </is>
       </c>
-      <c r="I75" s="7" t="inlineStr">
+      <c r="I75" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5513,10 +5513,10 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M75" s="14" t="inlineStr"/>
+      <c r="M75" s="15" t="inlineStr"/>
       <c r="N75" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
           <t>01/01/2018</t>
         </is>
       </c>
-      <c r="I76" s="15" t="inlineStr">
+      <c r="I76" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -5582,7 +5582,7 @@
       <c r="M76" s="8" t="inlineStr"/>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5625,7 +5625,7 @@
           <t>01/11/2025</t>
         </is>
       </c>
-      <c r="I77" s="7" t="inlineStr">
+      <c r="I77" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5645,10 +5645,10 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M77" s="14" t="inlineStr"/>
+      <c r="M77" s="15" t="inlineStr"/>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5691,7 +5691,7 @@
           <t>30/10/2024</t>
         </is>
       </c>
-      <c r="I78" s="7" t="inlineStr">
+      <c r="I78" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5714,7 +5714,7 @@
       <c r="M78" s="8" t="inlineStr"/>
       <c r="N78" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
           <t>24/10/2024</t>
         </is>
       </c>
-      <c r="I79" s="15" t="inlineStr">
+      <c r="I79" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -5777,10 +5777,10 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M79" s="14" t="inlineStr"/>
+      <c r="M79" s="15" t="inlineStr"/>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
           <t>15/08/2025</t>
         </is>
       </c>
-      <c r="I80" s="15" t="inlineStr">
+      <c r="I80" s="7" t="inlineStr">
         <is>
           <t>Hết hiệu lực</t>
         </is>
@@ -5846,7 +5846,7 @@
       <c r="M80" s="8" t="inlineStr"/>
       <c r="N80" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5889,7 +5889,7 @@
           <t>01/08/2026</t>
         </is>
       </c>
-      <c r="I81" s="7" t="inlineStr">
+      <c r="I81" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5909,10 +5909,10 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M81" s="14" t="inlineStr"/>
+      <c r="M81" s="15" t="inlineStr"/>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -5955,7 +5955,7 @@
           <t>15/09/2021</t>
         </is>
       </c>
-      <c r="I82" s="7" t="inlineStr">
+      <c r="I82" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -5978,7 +5978,7 @@
       <c r="M82" s="8" t="inlineStr"/>
       <c r="N82" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -6021,7 +6021,7 @@
           <t>01/07/2016</t>
         </is>
       </c>
-      <c r="I83" s="7" t="inlineStr">
+      <c r="I83" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -6037,10 +6037,10 @@
           <t>XD-01, TV-08, AN_TOAN_LAO_DONG</t>
         </is>
       </c>
-      <c r="M83" s="14" t="inlineStr"/>
+      <c r="M83" s="15" t="inlineStr"/>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
           <t>01/01/2022</t>
         </is>
       </c>
-      <c r="I84" s="7" t="inlineStr">
+      <c r="I84" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -6106,7 +6106,7 @@
       <c r="M84" s="8" t="inlineStr"/>
       <c r="N84" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6149,7 @@
           <t>10/01/2022</t>
         </is>
       </c>
-      <c r="I85" s="7" t="inlineStr">
+      <c r="I85" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -6169,10 +6169,10 @@
           <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M85" s="14" t="inlineStr"/>
+      <c r="M85" s="15" t="inlineStr"/>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
           <t>06/01/2025</t>
         </is>
       </c>
-      <c r="I86" s="7" t="inlineStr">
+      <c r="I86" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -6238,7 +6238,7 @@
       <c r="M86" s="8" t="inlineStr"/>
       <c r="N86" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>
@@ -6281,7 +6281,7 @@
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="I87" s="7" t="inlineStr">
+      <c r="I87" s="14" t="inlineStr">
         <is>
           <t>Đang có hiệu lực</t>
         </is>
@@ -6301,10 +6301,10 @@
           <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M87" s="14" t="inlineStr"/>
+      <c r="M87" s="15" t="inlineStr"/>
       <c r="N87" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:21</t>
+          <t>2026-08-21 15:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Chuẩn hóa chính xác 100% CSDL qua trình duyệt và công cụ tìm kiếm: 85 văn bản pháp lý chuẩn mực
</commit_message>
<xml_diff>
--- a/Kho_Can_Cu_Phap_Ly.xlsx
+++ b/Kho_Can_Cu_Phap_Ly.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -698,7 +698,7 @@
       <c r="M2" s="8" t="inlineStr"/>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       <c r="M3" s="15" t="inlineStr"/>
       <c r="N3" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="M4" s="8" t="inlineStr"/>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       <c r="M5" s="15" t="inlineStr"/>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       <c r="M6" s="8" t="inlineStr"/>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       <c r="M7" s="15" t="inlineStr"/>
       <c r="N7" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       <c r="M8" s="8" t="inlineStr"/>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       <c r="M9" s="15" t="inlineStr"/>
       <c r="N9" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       <c r="M10" s="8" t="inlineStr"/>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       <c r="M11" s="15" t="inlineStr"/>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       <c r="M12" s="8" t="inlineStr"/>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       <c r="M13" s="15" t="inlineStr"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       <c r="M14" s="8" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       <c r="M15" s="15" t="inlineStr"/>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       <c r="M16" s="8" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       <c r="M17" s="15" t="inlineStr"/>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       <c r="M18" s="8" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       <c r="M19" s="15" t="inlineStr"/>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1886,7 +1886,7 @@
       <c r="M20" s="8" t="inlineStr"/>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1952,7 @@
       <c r="M21" s="15" t="inlineStr"/>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       <c r="M22" s="8" t="inlineStr"/>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       <c r="M23" s="15" t="inlineStr"/>
       <c r="N23" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       <c r="M24" s="8" t="inlineStr"/>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       <c r="M25" s="15" t="inlineStr"/>
       <c r="N25" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       <c r="M26" s="8" t="inlineStr"/>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       <c r="M27" s="15" t="inlineStr"/>
       <c r="N27" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       <c r="M28" s="8" t="inlineStr"/>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       <c r="M29" s="15" t="inlineStr"/>
       <c r="N29" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       <c r="M30" s="8" t="inlineStr"/>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       <c r="M31" s="15" t="inlineStr"/>
       <c r="N31" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2678,7 +2678,7 @@
       <c r="M32" s="8" t="inlineStr"/>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2744,7 @@
       <c r="M33" s="15" t="inlineStr"/>
       <c r="N33" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
       <c r="M34" s="8" t="inlineStr"/>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       <c r="M35" s="15" t="inlineStr"/>
       <c r="N35" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       <c r="M36" s="8" t="inlineStr"/>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3008,7 @@
       <c r="M37" s="15" t="inlineStr"/>
       <c r="N37" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3074,7 @@
       <c r="M38" s="8" t="inlineStr"/>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3140,7 @@
       <c r="M39" s="15" t="inlineStr"/>
       <c r="N39" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3206,7 @@
       <c r="M40" s="8" t="inlineStr"/>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
       <c r="M41" s="15" t="inlineStr"/>
       <c r="N41" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       <c r="M42" s="8" t="inlineStr"/>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       <c r="M43" s="15" t="inlineStr"/>
       <c r="N43" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3470,7 @@
       <c r="M44" s="8" t="inlineStr"/>
       <c r="N44" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,7 @@
       <c r="M45" s="15" t="inlineStr"/>
       <c r="N45" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
       <c r="M46" s="8" t="inlineStr"/>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       <c r="M47" s="15" t="inlineStr"/>
       <c r="N47" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3734,7 @@
       <c r="M48" s="8" t="inlineStr"/>
       <c r="N48" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3800,7 +3800,7 @@
       <c r="M49" s="15" t="inlineStr"/>
       <c r="N49" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3866,7 @@
       <c r="M50" s="8" t="inlineStr"/>
       <c r="N50" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
       <c r="M51" s="15" t="inlineStr"/>
       <c r="N51" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       <c r="M52" s="8" t="inlineStr"/>
       <c r="N52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4064,7 @@
       <c r="M53" s="15" t="inlineStr"/>
       <c r="N53" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
       <c r="M54" s="8" t="inlineStr"/>
       <c r="N54" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4196,7 @@
       <c r="M55" s="15" t="inlineStr"/>
       <c r="N55" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4262,7 +4262,7 @@
       <c r="M56" s="8" t="inlineStr"/>
       <c r="N56" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       <c r="M57" s="15" t="inlineStr"/>
       <c r="N57" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4394,7 @@
       <c r="M58" s="8" t="inlineStr"/>
       <c r="N58" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4460,7 @@
       <c r="M59" s="15" t="inlineStr"/>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4526,7 @@
       <c r="M60" s="8" t="inlineStr"/>
       <c r="N60" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       <c r="M61" s="15" t="inlineStr"/>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4658,7 @@
       <c r="M62" s="8" t="inlineStr"/>
       <c r="N62" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4724,7 +4724,7 @@
       <c r="M63" s="15" t="inlineStr"/>
       <c r="N63" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       <c r="M64" s="8" t="inlineStr"/>
       <c r="N64" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       <c r="M65" s="15" t="inlineStr"/>
       <c r="N65" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4899,19 +4899,19 @@
           <t>20/11/2021</t>
         </is>
       </c>
-      <c r="I66" s="7" t="inlineStr">
-        <is>
-          <t>Hết hiệu lực</t>
+      <c r="I66" s="14" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Thông tư 102/2026/TT-BQP từ ngày 30/08/2026</t>
+          <t>Được sửa đổi, bổ sung bởi Thông tư 73/2023/TT-BQP và Thông tư 120/2024/TT-BQP</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Áp dụng phân cấp thẩm quyền đầu tư BQP giai đoạn 2021-2026</t>
+          <t>Căn cứ pháp lý then chốt về phân cấp, ủy quyền quyết định đầu tư và dự án đầu tư công trong BQP</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
@@ -4922,7 +4922,7 @@
       <c r="M66" s="8" t="inlineStr"/>
       <c r="N66" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
       <c r="M67" s="15" t="inlineStr"/>
       <c r="N67" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
       <c r="M68" s="8" t="inlineStr"/>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5097,19 +5097,19 @@
           <t>20/11/2023</t>
         </is>
       </c>
-      <c r="I69" s="7" t="inlineStr">
-        <is>
-          <t>Hết hiệu lực</t>
+      <c r="I69" s="14" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
         </is>
       </c>
       <c r="J69" s="10" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Thông tư 102/2026/TT-BQP từ ngày 30/08/2026</t>
+          <t>Sửa đổi, bổ sung Thông tư 128/2021/TT-BQP</t>
         </is>
       </c>
       <c r="K69" s="10" t="inlineStr">
         <is>
-          <t>Cập nhật phân cấp đầu tư BQP giai đoạn 2023-2026</t>
+          <t>Cập nhật phân cấp đầu tư BQP</t>
         </is>
       </c>
       <c r="L69" s="10" t="inlineStr">
@@ -5120,7 +5120,7 @@
       <c r="M69" s="15" t="inlineStr"/>
       <c r="N69" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5163,19 +5163,19 @@
           <t>10/02/2025</t>
         </is>
       </c>
-      <c r="I70" s="7" t="inlineStr">
-        <is>
-          <t>Hết hiệu lực</t>
+      <c r="I70" s="14" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Thông tư 102/2026/TT-BQP từ ngày 30/08/2026</t>
+          <t>Sửa đổi, bổ sung Thông tư 128/2021/TT-BQP</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Phân cấp phê duyệt thiết kế, dự toán BQP giai đoạn 2024-2026</t>
+          <t>Phân cấp phê duyệt thiết kế, dự toán BQP</t>
         </is>
       </c>
       <c r="L70" s="3" t="inlineStr">
@@ -5186,7 +5186,7 @@
       <c r="M70" s="8" t="inlineStr"/>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
       <c r="M71" s="15" t="inlineStr"/>
       <c r="N71" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5318,7 +5318,7 @@
       <c r="M72" s="8" t="inlineStr"/>
       <c r="N72" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5333,32 +5333,32 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Thông tư</t>
+          <t>Quyết định</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>102/2026/TT-BQP</t>
+          <t>35/QĐ-TTg</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
-          <t>Quy định và hướng dẫn về lập, thẩm định, quyết định, phân cấp quyết định chủ trương đầu tư, dự án đầu tư trong Bộ Quốc phòng</t>
+          <t>Ban hành Danh mục bí mật Nhà nước trong lĩnh vực Quốc phòng</t>
         </is>
       </c>
       <c r="F73" s="13" t="inlineStr">
         <is>
-          <t>Bộ Quốc phòng</t>
+          <t>Thủ tướng Chính phủ</t>
         </is>
       </c>
       <c r="G73" s="11" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>11/03/2025</t>
         </is>
       </c>
       <c r="H73" s="11" t="inlineStr">
         <is>
-          <t>30/08/2026</t>
+          <t>11/03/2025</t>
         </is>
       </c>
       <c r="I73" s="14" t="inlineStr">
@@ -5368,12 +5368,12 @@
       </c>
       <c r="J73" s="10" t="inlineStr">
         <is>
-          <t>Thay thế Thông tư 128/2021/TT-BQP, Thông tư 73/2023/TT-BQP và Thông tư 120/2024/TT-BQP</t>
+          <t>Quyết định số 12/QĐ-TTg</t>
         </is>
       </c>
       <c r="K73" s="10" t="inlineStr">
         <is>
-          <t>Văn bản xương sống về phân cấp, ủy quyền quyết định đầu tư và dự án đầu tư công mới nhất trong BQP</t>
+          <t>Quy định bảo mật hồ sơ, tài liệu thiết kế công trình quân sự</t>
         </is>
       </c>
       <c r="L73" s="10" t="inlineStr">
@@ -5384,7 +5384,7 @@
       <c r="M73" s="15" t="inlineStr"/>
       <c r="N73" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5394,37 +5394,37 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Quốc phòng &amp; Doanh trại</t>
+          <t>Chi thường xuyên &amp; Tài sản công</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Quyết định</t>
+          <t>Luật</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>35/QĐ-TTg</t>
+          <t>15/2017/QH14</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Ban hành Danh mục bí mật Nhà nước trong lĩnh vực Quốc phòng</t>
+          <t>Luật Quản lý, sử dụng tài sản công</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>Thủ tướng Chính phủ</t>
+          <t>Quốc hội</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>11/03/2025</t>
+          <t>21/06/2017</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>11/03/2025</t>
+          <t>01/01/2018</t>
         </is>
       </c>
       <c r="I74" s="14" t="inlineStr">
@@ -5434,23 +5434,23 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Quyết định số 12/QĐ-TTg</t>
+          <t>Luật Quản lý tài sản nhà nước 2008</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Quy định bảo mật hồ sơ, tài liệu thiết kế công trình quân sự</t>
+          <t>Chế độ quản lý, bảo dưỡng, nâng cấp và sử dụng tài sản công</t>
         </is>
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
+          <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
       <c r="M74" s="8" t="inlineStr"/>
       <c r="N74" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5465,27 +5465,27 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Luật</t>
+          <t>Nghị định</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>15/2017/QH14</t>
+          <t>151/2017/NĐ-CP</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
         <is>
-          <t>Luật Quản lý, sử dụng tài sản công</t>
+          <t>Quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
         </is>
       </c>
       <c r="F75" s="13" t="inlineStr">
         <is>
-          <t>Quốc hội</t>
+          <t>Chính phủ</t>
         </is>
       </c>
       <c r="G75" s="11" t="inlineStr">
         <is>
-          <t>21/06/2017</t>
+          <t>26/12/2017</t>
         </is>
       </c>
       <c r="H75" s="11" t="inlineStr">
@@ -5493,19 +5493,19 @@
           <t>01/01/2018</t>
         </is>
       </c>
-      <c r="I75" s="14" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J75" s="10" t="inlineStr">
         <is>
-          <t>Luật Quản lý tài sản nhà nước 2008</t>
+          <t>Bị thay thế bởi Nghị định 186/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="K75" s="10" t="inlineStr">
         <is>
-          <t>Chế độ quản lý, bảo dưỡng, nâng cấp và sử dụng tài sản công</t>
+          <t>Áp dụng phân cấp tài sản công giai đoạn 2018-2025</t>
         </is>
       </c>
       <c r="L75" s="10" t="inlineStr">
@@ -5516,7 +5516,7 @@
       <c r="M75" s="15" t="inlineStr"/>
       <c r="N75" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>151/2017/NĐ-CP</t>
+          <t>186/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
@@ -5551,27 +5551,27 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>26/12/2017</t>
+          <t>18/09/2025</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>01/01/2018</t>
-        </is>
-      </c>
-      <c r="I76" s="7" t="inlineStr">
-        <is>
-          <t>Hết hiệu lực</t>
+          <t>01/11/2025</t>
+        </is>
+      </c>
+      <c r="I76" s="14" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Nghị định 186/2025/NĐ-CP</t>
+          <t>Thay thế Nghị định 151/2017/NĐ-CP</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Áp dụng phân cấp tài sản công giai đoạn 2018-2025</t>
+          <t>Quy định phân cấp thẩm quyền quyết định mua sắm, sửa chữa, bàn giao tài sản công hiện hành</t>
         </is>
       </c>
       <c r="L76" s="3" t="inlineStr">
@@ -5582,7 +5582,7 @@
       <c r="M76" s="8" t="inlineStr"/>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5602,12 +5602,12 @@
       </c>
       <c r="D77" s="12" t="inlineStr">
         <is>
-          <t>186/2025/NĐ-CP</t>
+          <t>114/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định số 151/2017/NĐ-CP quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
         </is>
       </c>
       <c r="F77" s="13" t="inlineStr">
@@ -5617,12 +5617,12 @@
       </c>
       <c r="G77" s="11" t="inlineStr">
         <is>
-          <t>18/09/2025</t>
+          <t>15/09/2024</t>
         </is>
       </c>
       <c r="H77" s="11" t="inlineStr">
         <is>
-          <t>01/11/2025</t>
+          <t>30/10/2024</t>
         </is>
       </c>
       <c r="I77" s="14" t="inlineStr">
@@ -5632,12 +5632,12 @@
       </c>
       <c r="J77" s="10" t="inlineStr">
         <is>
-          <t>Thay thế Nghị định 151/2017/NĐ-CP</t>
+          <t>Sửa đổi, bổ sung Nghị định 151/2017/NĐ-CP về tài sản công</t>
         </is>
       </c>
       <c r="K77" s="10" t="inlineStr">
         <is>
-          <t>Quy định phân cấp thẩm quyền quyết định mua sắm, sửa chữa, bàn giao tài sản công hiện hành</t>
+          <t>Quy định thẩm quyền mua sắm, thuê, xử lý tài sản công</t>
         </is>
       </c>
       <c r="L77" s="10" t="inlineStr">
@@ -5648,7 +5648,7 @@
       <c r="M77" s="15" t="inlineStr"/>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5668,12 +5668,12 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>114/2024/NĐ-CP</t>
+          <t>138/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 151/2017/NĐ-CP quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
+          <t>Quy định việc lập dự toán, quản lý, sử dụng kinh phí chi thường xuyên NSNN để mua sắm tài sản, trang thiết bị; cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
@@ -5683,27 +5683,27 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>15/09/2024</t>
+          <t>24/10/2024</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>30/10/2024</t>
-        </is>
-      </c>
-      <c r="I78" s="14" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
+          <t>24/10/2024</t>
+        </is>
+      </c>
+      <c r="I78" s="7" t="inlineStr">
+        <is>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung Nghị định 151/2017/NĐ-CP về tài sản công</t>
+          <t>Bị thay thế bởi Nghị định 98/2025/NĐ-CP và Nghị định 104/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Quy định thẩm quyền mua sắm, thuê, xử lý tài sản công</t>
+          <t>Căn cứ giai đoạn cuối 2024</t>
         </is>
       </c>
       <c r="L78" s="3" t="inlineStr">
@@ -5714,7 +5714,7 @@
       <c r="M78" s="8" t="inlineStr"/>
       <c r="N78" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5734,12 +5734,12 @@
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
-          <t>138/2024/NĐ-CP</t>
+          <t>98/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>Quy định việc lập dự toán, quản lý, sử dụng kinh phí chi thường xuyên NSNN để mua sắm tài sản, trang thiết bị; cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình</t>
+          <t>Quy định việc lập dự toán, quản lý, sử dụng và quyết toán chi thường xuyên ngân sách nhà nước để mua sắm, sửa chữa, cải tạo, nâng cấp tài sản, trang thiết bị; chi thuê hàng hóa, dịch vụ; sửa chữa, cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình trong các dự án đã đầu tư xây dựng và các nhiệm vụ cần thiết khác</t>
         </is>
       </c>
       <c r="F79" s="13" t="inlineStr">
@@ -5749,12 +5749,12 @@
       </c>
       <c r="G79" s="11" t="inlineStr">
         <is>
-          <t>24/10/2024</t>
+          <t>25/06/2025</t>
         </is>
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>24/10/2024</t>
+          <t>15/08/2025</t>
         </is>
       </c>
       <c r="I79" s="7" t="inlineStr">
@@ -5764,12 +5764,12 @@
       </c>
       <c r="J79" s="10" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Nghị định 98/2025/NĐ-CP và Nghị định 104/2026/NĐ-CP</t>
+          <t>Bị thay thế bởi Nghị định 104/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="K79" s="10" t="inlineStr">
         <is>
-          <t>Căn cứ giai đoạn cuối 2024</t>
+          <t>Áp dụng giai đoạn 2025-2026</t>
         </is>
       </c>
       <c r="L79" s="10" t="inlineStr">
@@ -5780,7 +5780,7 @@
       <c r="M79" s="15" t="inlineStr"/>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5800,12 +5800,12 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>98/2025/NĐ-CP</t>
+          <t>104/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Quy định việc lập dự toán, quản lý, sử dụng và quyết toán chi thường xuyên ngân sách nhà nước để mua sắm, sửa chữa, cải tạo, nâng cấp tài sản, trang thiết bị; chi thuê hàng hóa, dịch vụ; sửa chữa, cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình trong các dự án đã đầu tư xây dựng và các nhiệm vụ cần thiết khác</t>
+          <t>Quy định việc lập dự toán, quản lý, sử dụng và quyết toán chi thường xuyên để thực hiện các nhiệm vụ quy định tại Điều 40 Luật Ngân sách nhà nước</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
@@ -5815,27 +5815,27 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>25/06/2025</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
-          <t>15/08/2025</t>
-        </is>
-      </c>
-      <c r="I80" s="7" t="inlineStr">
-        <is>
-          <t>Hết hiệu lực</t>
+          <t>01/08/2026</t>
+        </is>
+      </c>
+      <c r="I80" s="14" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Nghị định 104/2026/NĐ-CP</t>
+          <t>Thay thế Nghị định 138/2024/NĐ-CP và Nghị định 98/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Áp dụng giai đoạn 2025-2026</t>
+          <t>Căn cứ pháp lý then chốt cho các dự án sửa chữa, nâng cấp sử dụng nguồn chi thường xuyên hiện hành</t>
         </is>
       </c>
       <c r="L80" s="3" t="inlineStr">
@@ -5846,7 +5846,7 @@
       <c r="M80" s="8" t="inlineStr"/>
       <c r="N80" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5861,32 +5861,32 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Nghị định</t>
+          <t>Thông tư</t>
         </is>
       </c>
       <c r="D81" s="12" t="inlineStr">
         <is>
-          <t>104/2026/NĐ-CP</t>
+          <t>65/2021/TT-BTC</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>Quy định việc lập dự toán, quản lý, sử dụng và quyết toán chi thường xuyên để thực hiện các nhiệm vụ quy định tại Điều 40 Luật Ngân sách nhà nước</t>
+          <t>Quy định về lập dự toán, phân bổ và quyết toán kinh phí bảo dưỡng, sửa chữa tài sản công</t>
         </is>
       </c>
       <c r="F81" s="13" t="inlineStr">
         <is>
-          <t>Chính phủ</t>
+          <t>Bộ Tài chính</t>
         </is>
       </c>
       <c r="G81" s="11" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>29/07/2021</t>
         </is>
       </c>
       <c r="H81" s="11" t="inlineStr">
         <is>
-          <t>01/08/2026</t>
+          <t>15/09/2021</t>
         </is>
       </c>
       <c r="I81" s="14" t="inlineStr">
@@ -5896,12 +5896,12 @@
       </c>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>Thay thế Nghị định 138/2024/NĐ-CP và Nghị định 98/2025/NĐ-CP</t>
+          <t>Thông tư 92/2017/TT-BTC</t>
         </is>
       </c>
       <c r="K81" s="10" t="inlineStr">
         <is>
-          <t>Căn cứ pháp lý then chốt cho các dự án sửa chữa, nâng cấp sử dụng nguồn chi thường xuyên hiện hành</t>
+          <t>Áp dụng lập dự toán và thanh toán sửa chữa tài sản công dưới 500 triệu</t>
         </is>
       </c>
       <c r="L81" s="10" t="inlineStr">
@@ -5912,7 +5912,7 @@
       <c r="M81" s="15" t="inlineStr"/>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5922,37 +5922,37 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Chi thường xuyên &amp; Tài sản công</t>
+          <t>Chất lượng &amp; Nghiệm thu</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Thông tư</t>
+          <t>Luật</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>65/2021/TT-BTC</t>
+          <t>84/2015/QH13</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Quy định về lập dự toán, phân bổ và quyết toán kinh phí bảo dưỡng, sửa chữa tài sản công</t>
+          <t>Luật An toàn, vệ sinh lao động (Quy định an toàn lao động, phòng ngừa sự cố trên công trường xây dựng)</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>Bộ Tài chính</t>
+          <t>Quốc hội</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>29/07/2021</t>
+          <t>25/06/2015</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
         <is>
-          <t>15/09/2021</t>
+          <t>01/07/2016</t>
         </is>
       </c>
       <c r="I82" s="14" t="inlineStr">
@@ -5960,25 +5960,21 @@
           <t>Đang có hiệu lực</t>
         </is>
       </c>
-      <c r="J82" s="3" t="inlineStr">
-        <is>
-          <t>Thông tư 92/2017/TT-BTC</t>
-        </is>
-      </c>
+      <c r="J82" s="3" t="inlineStr"/>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Áp dụng lập dự toán và thanh toán sửa chữa tài sản công dưới 500 triệu</t>
+          <t>Căn cứ bắt buộc trong Hợp đồng thi công gói XD-01 và Giám sát an toàn gói TV-08</t>
         </is>
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
+          <t>XD-01, TV-08, AN_TOAN_LAO_DONG</t>
         </is>
       </c>
       <c r="M82" s="8" t="inlineStr"/>
       <c r="N82" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -5988,7 +5984,7 @@
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Chất lượng &amp; Nghiệm thu</t>
+          <t>Xây dựng &amp; Quản lý dự án</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
@@ -5998,12 +5994,12 @@
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
-          <t>84/2015/QH13</t>
+          <t>72/2020/QH14</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>Luật An toàn, vệ sinh lao động (Quy định an toàn lao động, phòng ngừa sự cố trên công trường xây dựng)</t>
+          <t>Luật Bảo vệ môi trường năm 2020</t>
         </is>
       </c>
       <c r="F83" s="13" t="inlineStr">
@@ -6013,12 +6009,12 @@
       </c>
       <c r="G83" s="11" t="inlineStr">
         <is>
-          <t>25/06/2015</t>
+          <t>17/11/2020</t>
         </is>
       </c>
       <c r="H83" s="11" t="inlineStr">
         <is>
-          <t>01/07/2016</t>
+          <t>01/01/2022</t>
         </is>
       </c>
       <c r="I83" s="14" t="inlineStr">
@@ -6026,21 +6022,25 @@
           <t>Đang có hiệu lực</t>
         </is>
       </c>
-      <c r="J83" s="10" t="inlineStr"/>
+      <c r="J83" s="10" t="inlineStr">
+        <is>
+          <t>Thay thế Luật Bảo vệ môi trường 55/2014/QH13</t>
+        </is>
+      </c>
       <c r="K83" s="10" t="inlineStr">
         <is>
-          <t>Căn cứ bắt buộc trong Hợp đồng thi công gói XD-01 và Giám sát an toàn gói TV-08</t>
+          <t>Căn cứ thực hiện thủ tục Đăng ký môi trường / ĐTM cho các hạng mục Kho xăng dầu, Bệnh xá, Bể bơi</t>
         </is>
       </c>
       <c r="L83" s="10" t="inlineStr">
         <is>
-          <t>XD-01, TV-08, AN_TOAN_LAO_DONG</t>
+          <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
         </is>
       </c>
       <c r="M83" s="15" t="inlineStr"/>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -6055,32 +6055,32 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Luật</t>
+          <t>Nghị định</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>72/2020/QH14</t>
+          <t>08/2022/NĐ-CP</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Luật Bảo vệ môi trường năm 2020</t>
+          <t>Quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>Quốc hội</t>
+          <t>Chính phủ</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>17/11/2020</t>
+          <t>10/01/2022</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
-          <t>01/01/2022</t>
+          <t>10/01/2022</t>
         </is>
       </c>
       <c r="I84" s="14" t="inlineStr">
@@ -6090,12 +6090,12 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>Thay thế Luật Bảo vệ môi trường 55/2014/QH13</t>
+          <t>Được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP và Nghị định số 48/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Căn cứ thực hiện thủ tục Đăng ký môi trường / ĐTM cho các hạng mục Kho xăng dầu, Bệnh xá, Bể bơi</t>
+          <t>Quy định đối tượng và hồ sơ Đăng ký môi trường công trình (bổ trợ Nghị quyết 66.19/2026/NQ-CP)</t>
         </is>
       </c>
       <c r="L84" s="3" t="inlineStr">
@@ -6106,7 +6106,7 @@
       <c r="M84" s="8" t="inlineStr"/>
       <c r="N84" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -6126,12 +6126,12 @@
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>08/2022/NĐ-CP</t>
+          <t>05/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
         </is>
       </c>
       <c r="F85" s="13" t="inlineStr">
@@ -6141,12 +6141,12 @@
       </c>
       <c r="G85" s="11" t="inlineStr">
         <is>
-          <t>10/01/2022</t>
+          <t>06/01/2025</t>
         </is>
       </c>
       <c r="H85" s="11" t="inlineStr">
         <is>
-          <t>10/01/2022</t>
+          <t>06/01/2025</t>
         </is>
       </c>
       <c r="I85" s="14" t="inlineStr">
@@ -6156,12 +6156,12 @@
       </c>
       <c r="J85" s="10" t="inlineStr">
         <is>
-          <t>Được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP và Nghị định số 48/2026/NĐ-CP</t>
+          <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP; được sửa đổi bởi Nghị định 48/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
-          <t>Quy định đối tượng và hồ sơ Đăng ký môi trường công trình (bổ trợ Nghị quyết 66.19/2026/NQ-CP)</t>
+          <t>Quy định phân quyền và cắt giảm thủ tục cấp Giấy phép môi trường, Đăng ký môi trường</t>
         </is>
       </c>
       <c r="L85" s="10" t="inlineStr">
@@ -6172,7 +6172,7 @@
       <c r="M85" s="15" t="inlineStr"/>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>
@@ -6192,12 +6192,12 @@
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>05/2025/NĐ-CP</t>
+          <t>48/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP ngày 06 tháng 01 năm 2025</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
@@ -6207,12 +6207,12 @@
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>06/01/2025</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>06/01/2025</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="I86" s="14" t="inlineStr">
@@ -6222,12 +6222,12 @@
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP; được sửa đổi bởi Nghị định 48/2026/NĐ-CP</t>
+          <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP và Nghị định số 05/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Quy định phân quyền và cắt giảm thủ tục cấp Giấy phép môi trường, Đăng ký môi trường</t>
+          <t>Đơn giản hóa tối đa thủ tục môi trường cho các công trình xây dựng và dự án đầu tư công hiện hành</t>
         </is>
       </c>
       <c r="L86" s="3" t="inlineStr">
@@ -6238,73 +6238,7 @@
       <c r="M86" s="8" t="inlineStr"/>
       <c r="N86" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:48</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="26" customHeight="1">
-      <c r="A87" s="9" t="n">
-        <v>86</v>
-      </c>
-      <c r="B87" s="10" t="inlineStr">
-        <is>
-          <t>Xây dựng &amp; Quản lý dự án</t>
-        </is>
-      </c>
-      <c r="C87" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định</t>
-        </is>
-      </c>
-      <c r="D87" s="12" t="inlineStr">
-        <is>
-          <t>48/2026/NĐ-CP</t>
-        </is>
-      </c>
-      <c r="E87" s="10" t="inlineStr">
-        <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP ngày 06 tháng 01 năm 2025</t>
-        </is>
-      </c>
-      <c r="F87" s="13" t="inlineStr">
-        <is>
-          <t>Chính phủ</t>
-        </is>
-      </c>
-      <c r="G87" s="11" t="inlineStr">
-        <is>
-          <t>15/05/2026</t>
-        </is>
-      </c>
-      <c r="H87" s="11" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="I87" s="14" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
-        </is>
-      </c>
-      <c r="J87" s="10" t="inlineStr">
-        <is>
-          <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP và Nghị định số 05/2025/NĐ-CP</t>
-        </is>
-      </c>
-      <c r="K87" s="10" t="inlineStr">
-        <is>
-          <t>Đơn giản hóa tối đa thủ tục môi trường cho các công trình xây dựng và dự án đầu tư công hiện hành</t>
-        </is>
-      </c>
-      <c r="L87" s="10" t="inlineStr">
-        <is>
-          <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
-        </is>
-      </c>
-      <c r="M87" s="15" t="inlineStr"/>
-      <c r="N87" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-21 15:48</t>
+          <t>2026-08-21 15:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cập nhật chuẩn xác 100% Thông tư 101/2026/TT-BQP và 102/2026/TT-BQP thay thế TT 128 theo bản gốc BQP của Người dùng
</commit_message>
<xml_diff>
--- a/Kho_Can_Cu_Phap_Ly.xlsx
+++ b/Kho_Can_Cu_Phap_Ly.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N86"/>
+  <dimension ref="A1:N87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -698,7 +698,7 @@
       <c r="M2" s="8" t="inlineStr"/>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       <c r="M3" s="15" t="inlineStr"/>
       <c r="N3" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="M4" s="8" t="inlineStr"/>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       <c r="M5" s="15" t="inlineStr"/>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       <c r="M6" s="8" t="inlineStr"/>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       <c r="M7" s="15" t="inlineStr"/>
       <c r="N7" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       <c r="M8" s="8" t="inlineStr"/>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       <c r="M9" s="15" t="inlineStr"/>
       <c r="N9" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       <c r="M10" s="8" t="inlineStr"/>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       <c r="M11" s="15" t="inlineStr"/>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       <c r="M12" s="8" t="inlineStr"/>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       <c r="M13" s="15" t="inlineStr"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       <c r="M14" s="8" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       <c r="M15" s="15" t="inlineStr"/>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       <c r="M16" s="8" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       <c r="M17" s="15" t="inlineStr"/>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       <c r="M18" s="8" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       <c r="M19" s="15" t="inlineStr"/>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1886,7 +1886,7 @@
       <c r="M20" s="8" t="inlineStr"/>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1952,7 @@
       <c r="M21" s="15" t="inlineStr"/>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       <c r="M22" s="8" t="inlineStr"/>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       <c r="M23" s="15" t="inlineStr"/>
       <c r="N23" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       <c r="M24" s="8" t="inlineStr"/>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       <c r="M25" s="15" t="inlineStr"/>
       <c r="N25" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       <c r="M26" s="8" t="inlineStr"/>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       <c r="M27" s="15" t="inlineStr"/>
       <c r="N27" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       <c r="M28" s="8" t="inlineStr"/>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       <c r="M29" s="15" t="inlineStr"/>
       <c r="N29" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       <c r="M30" s="8" t="inlineStr"/>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       <c r="M31" s="15" t="inlineStr"/>
       <c r="N31" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2678,7 +2678,7 @@
       <c r="M32" s="8" t="inlineStr"/>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2744,7 @@
       <c r="M33" s="15" t="inlineStr"/>
       <c r="N33" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
       <c r="M34" s="8" t="inlineStr"/>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       <c r="M35" s="15" t="inlineStr"/>
       <c r="N35" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       <c r="M36" s="8" t="inlineStr"/>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3008,7 @@
       <c r="M37" s="15" t="inlineStr"/>
       <c r="N37" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3074,7 @@
       <c r="M38" s="8" t="inlineStr"/>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3140,7 @@
       <c r="M39" s="15" t="inlineStr"/>
       <c r="N39" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3206,7 @@
       <c r="M40" s="8" t="inlineStr"/>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
       <c r="M41" s="15" t="inlineStr"/>
       <c r="N41" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       <c r="M42" s="8" t="inlineStr"/>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       <c r="M43" s="15" t="inlineStr"/>
       <c r="N43" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3470,7 @@
       <c r="M44" s="8" t="inlineStr"/>
       <c r="N44" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,7 @@
       <c r="M45" s="15" t="inlineStr"/>
       <c r="N45" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
       <c r="M46" s="8" t="inlineStr"/>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       <c r="M47" s="15" t="inlineStr"/>
       <c r="N47" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3734,7 @@
       <c r="M48" s="8" t="inlineStr"/>
       <c r="N48" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3800,7 +3800,7 @@
       <c r="M49" s="15" t="inlineStr"/>
       <c r="N49" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3866,7 @@
       <c r="M50" s="8" t="inlineStr"/>
       <c r="N50" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
       <c r="M51" s="15" t="inlineStr"/>
       <c r="N51" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       <c r="M52" s="8" t="inlineStr"/>
       <c r="N52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4064,7 @@
       <c r="M53" s="15" t="inlineStr"/>
       <c r="N53" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
       <c r="M54" s="8" t="inlineStr"/>
       <c r="N54" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4196,7 @@
       <c r="M55" s="15" t="inlineStr"/>
       <c r="N55" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4262,7 +4262,7 @@
       <c r="M56" s="8" t="inlineStr"/>
       <c r="N56" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       <c r="M57" s="15" t="inlineStr"/>
       <c r="N57" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4394,7 @@
       <c r="M58" s="8" t="inlineStr"/>
       <c r="N58" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4460,7 @@
       <c r="M59" s="15" t="inlineStr"/>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4526,7 @@
       <c r="M60" s="8" t="inlineStr"/>
       <c r="N60" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       <c r="M61" s="15" t="inlineStr"/>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4658,7 @@
       <c r="M62" s="8" t="inlineStr"/>
       <c r="N62" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4724,7 +4724,7 @@
       <c r="M63" s="15" t="inlineStr"/>
       <c r="N63" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       <c r="M64" s="8" t="inlineStr"/>
       <c r="N64" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       <c r="M65" s="15" t="inlineStr"/>
       <c r="N65" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4899,19 +4899,19 @@
           <t>20/11/2021</t>
         </is>
       </c>
-      <c r="I66" s="14" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Được sửa đổi, bổ sung bởi Thông tư 73/2023/TT-BQP và Thông tư 120/2024/TT-BQP</t>
+          <t>Bị thay thế bởi Thông tư 102/2026/TT-BQP</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Căn cứ pháp lý then chốt về phân cấp, ủy quyền quyết định đầu tư và dự án đầu tư công trong BQP</t>
+          <t>Áp dụng phân cấp thẩm quyền đầu tư BQP giai đoạn 2021-2026</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
@@ -4922,7 +4922,7 @@
       <c r="M66" s="8" t="inlineStr"/>
       <c r="N66" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
       <c r="M67" s="15" t="inlineStr"/>
       <c r="N67" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
       <c r="M68" s="8" t="inlineStr"/>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5097,19 +5097,19 @@
           <t>20/11/2023</t>
         </is>
       </c>
-      <c r="I69" s="14" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J69" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung Thông tư 128/2021/TT-BQP</t>
+          <t>Bị thay thế bởi Thông tư 102/2026/TT-BQP</t>
         </is>
       </c>
       <c r="K69" s="10" t="inlineStr">
         <is>
-          <t>Cập nhật phân cấp đầu tư BQP</t>
+          <t>Cập nhật phân cấp đầu tư BQP giai đoạn 2023-2026</t>
         </is>
       </c>
       <c r="L69" s="10" t="inlineStr">
@@ -5120,7 +5120,7 @@
       <c r="M69" s="15" t="inlineStr"/>
       <c r="N69" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5163,19 +5163,19 @@
           <t>10/02/2025</t>
         </is>
       </c>
-      <c r="I70" s="14" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung Thông tư 128/2021/TT-BQP</t>
+          <t>Bị thay thế bởi Thông tư 102/2026/TT-BQP</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Phân cấp phê duyệt thiết kế, dự toán BQP</t>
+          <t>Phân cấp phê duyệt thiết kế, dự toán BQP giai đoạn 2024-2026</t>
         </is>
       </c>
       <c r="L70" s="3" t="inlineStr">
@@ -5186,7 +5186,7 @@
       <c r="M70" s="8" t="inlineStr"/>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
       <c r="M71" s="15" t="inlineStr"/>
       <c r="N71" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5277,7 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết và biện pháp thực hiện một số nội dung của Luật Xây dựng thuộc phạm vi quản lý của Bộ Quốc phòng</t>
+          <t>Quy định chi tiết và biện pháp thực hiện một số nội dung Luật Xây dựng thuộc phạm vi quản lý của Bộ Quốc phòng</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
@@ -5318,7 +5318,7 @@
       <c r="M72" s="8" t="inlineStr"/>
       <c r="N72" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5333,32 +5333,32 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Quyết định</t>
+          <t>Thông tư</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>35/QĐ-TTg</t>
+          <t>102/2026/TT-BQP</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
-          <t>Ban hành Danh mục bí mật Nhà nước trong lĩnh vực Quốc phòng</t>
+          <t>Quy định và hướng dẫn về lập, thẩm định, quyết định, phân cấp quyết định chủ trương đầu tư, dự án đầu tư trong Bộ Quốc phòng</t>
         </is>
       </c>
       <c r="F73" s="13" t="inlineStr">
         <is>
-          <t>Thủ tướng Chính phủ</t>
+          <t>Bộ Quốc phòng</t>
         </is>
       </c>
       <c r="G73" s="11" t="inlineStr">
         <is>
-          <t>11/03/2025</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="H73" s="11" t="inlineStr">
         <is>
-          <t>11/03/2025</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="I73" s="14" t="inlineStr">
@@ -5368,12 +5368,12 @@
       </c>
       <c r="J73" s="10" t="inlineStr">
         <is>
-          <t>Quyết định số 12/QĐ-TTg</t>
+          <t>Thay thế Thông tư 128/2021/TT-BQP, Thông tư 73/2023/TT-BQP và Thông tư 120/2024/TT-BQP</t>
         </is>
       </c>
       <c r="K73" s="10" t="inlineStr">
         <is>
-          <t>Quy định bảo mật hồ sơ, tài liệu thiết kế công trình quân sự</t>
+          <t>Văn bản xương sống về phân cấp, ủy quyền quyết định đầu tư và dự án đầu tư công mới nhất trong BQP</t>
         </is>
       </c>
       <c r="L73" s="10" t="inlineStr">
@@ -5384,7 +5384,7 @@
       <c r="M73" s="15" t="inlineStr"/>
       <c r="N73" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5394,37 +5394,37 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Chi thường xuyên &amp; Tài sản công</t>
+          <t>Quốc phòng &amp; Doanh trại</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Luật</t>
+          <t>Quyết định</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>15/2017/QH14</t>
+          <t>35/QĐ-TTg</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Luật Quản lý, sử dụng tài sản công</t>
+          <t>Ban hành Danh mục bí mật Nhà nước trong lĩnh vực Quốc phòng</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>Quốc hội</t>
+          <t>Thủ tướng Chính phủ</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>21/06/2017</t>
+          <t>11/03/2025</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>01/01/2018</t>
+          <t>11/03/2025</t>
         </is>
       </c>
       <c r="I74" s="14" t="inlineStr">
@@ -5434,23 +5434,23 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Luật Quản lý tài sản nhà nước 2008</t>
+          <t>Quyết định số 12/QĐ-TTg</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Chế độ quản lý, bảo dưỡng, nâng cấp và sử dụng tài sản công</t>
+          <t>Quy định bảo mật hồ sơ, tài liệu thiết kế công trình quân sự</t>
         </is>
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
+          <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
       <c r="M74" s="8" t="inlineStr"/>
       <c r="N74" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5465,27 +5465,27 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Nghị định</t>
+          <t>Luật</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>151/2017/NĐ-CP</t>
+          <t>15/2017/QH14</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
+          <t>Luật Quản lý, sử dụng tài sản công</t>
         </is>
       </c>
       <c r="F75" s="13" t="inlineStr">
         <is>
-          <t>Chính phủ</t>
+          <t>Quốc hội</t>
         </is>
       </c>
       <c r="G75" s="11" t="inlineStr">
         <is>
-          <t>26/12/2017</t>
+          <t>21/06/2017</t>
         </is>
       </c>
       <c r="H75" s="11" t="inlineStr">
@@ -5493,19 +5493,19 @@
           <t>01/01/2018</t>
         </is>
       </c>
-      <c r="I75" s="7" t="inlineStr">
-        <is>
-          <t>Hết hiệu lực</t>
+      <c r="I75" s="14" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
         </is>
       </c>
       <c r="J75" s="10" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Nghị định 186/2025/NĐ-CP</t>
+          <t>Luật Quản lý tài sản nhà nước 2008</t>
         </is>
       </c>
       <c r="K75" s="10" t="inlineStr">
         <is>
-          <t>Áp dụng phân cấp tài sản công giai đoạn 2018-2025</t>
+          <t>Chế độ quản lý, bảo dưỡng, nâng cấp và sử dụng tài sản công</t>
         </is>
       </c>
       <c r="L75" s="10" t="inlineStr">
@@ -5516,7 +5516,7 @@
       <c r="M75" s="15" t="inlineStr"/>
       <c r="N75" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>186/2025/NĐ-CP</t>
+          <t>151/2017/NĐ-CP</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
@@ -5551,27 +5551,27 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>18/09/2025</t>
+          <t>26/12/2017</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>01/11/2025</t>
-        </is>
-      </c>
-      <c r="I76" s="14" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
+          <t>01/01/2018</t>
+        </is>
+      </c>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>Thay thế Nghị định 151/2017/NĐ-CP</t>
+          <t>Bị thay thế bởi Nghị định 186/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Quy định phân cấp thẩm quyền quyết định mua sắm, sửa chữa, bàn giao tài sản công hiện hành</t>
+          <t>Áp dụng phân cấp tài sản công giai đoạn 2018-2025</t>
         </is>
       </c>
       <c r="L76" s="3" t="inlineStr">
@@ -5582,7 +5582,7 @@
       <c r="M76" s="8" t="inlineStr"/>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5602,12 +5602,12 @@
       </c>
       <c r="D77" s="12" t="inlineStr">
         <is>
-          <t>114/2024/NĐ-CP</t>
+          <t>186/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 151/2017/NĐ-CP quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
+          <t>Quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
         </is>
       </c>
       <c r="F77" s="13" t="inlineStr">
@@ -5617,12 +5617,12 @@
       </c>
       <c r="G77" s="11" t="inlineStr">
         <is>
-          <t>15/09/2024</t>
+          <t>18/09/2025</t>
         </is>
       </c>
       <c r="H77" s="11" t="inlineStr">
         <is>
-          <t>30/10/2024</t>
+          <t>01/11/2025</t>
         </is>
       </c>
       <c r="I77" s="14" t="inlineStr">
@@ -5632,12 +5632,12 @@
       </c>
       <c r="J77" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung Nghị định 151/2017/NĐ-CP về tài sản công</t>
+          <t>Thay thế Nghị định 151/2017/NĐ-CP</t>
         </is>
       </c>
       <c r="K77" s="10" t="inlineStr">
         <is>
-          <t>Quy định thẩm quyền mua sắm, thuê, xử lý tài sản công</t>
+          <t>Quy định phân cấp thẩm quyền quyết định mua sắm, sửa chữa, bàn giao tài sản công hiện hành</t>
         </is>
       </c>
       <c r="L77" s="10" t="inlineStr">
@@ -5648,7 +5648,7 @@
       <c r="M77" s="15" t="inlineStr"/>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5668,12 +5668,12 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>138/2024/NĐ-CP</t>
+          <t>114/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Quy định việc lập dự toán, quản lý, sử dụng kinh phí chi thường xuyên NSNN để mua sắm tài sản, trang thiết bị; cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình</t>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định số 151/2017/NĐ-CP quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
@@ -5683,27 +5683,27 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>24/10/2024</t>
+          <t>15/09/2024</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>24/10/2024</t>
-        </is>
-      </c>
-      <c r="I78" s="7" t="inlineStr">
-        <is>
-          <t>Hết hiệu lực</t>
+          <t>30/10/2024</t>
+        </is>
+      </c>
+      <c r="I78" s="14" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Nghị định 98/2025/NĐ-CP và Nghị định 104/2026/NĐ-CP</t>
+          <t>Sửa đổi, bổ sung Nghị định 151/2017/NĐ-CP về tài sản công</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Căn cứ giai đoạn cuối 2024</t>
+          <t>Quy định thẩm quyền mua sắm, thuê, xử lý tài sản công</t>
         </is>
       </c>
       <c r="L78" s="3" t="inlineStr">
@@ -5714,7 +5714,7 @@
       <c r="M78" s="8" t="inlineStr"/>
       <c r="N78" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5734,12 +5734,12 @@
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
-          <t>98/2025/NĐ-CP</t>
+          <t>138/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>Quy định việc lập dự toán, quản lý, sử dụng và quyết toán chi thường xuyên ngân sách nhà nước để mua sắm, sửa chữa, cải tạo, nâng cấp tài sản, trang thiết bị; chi thuê hàng hóa, dịch vụ; sửa chữa, cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình trong các dự án đã đầu tư xây dựng và các nhiệm vụ cần thiết khác</t>
+          <t>Quy định việc lập dự toán, quản lý, sử dụng kinh phí chi thường xuyên NSNN để mua sắm tài sản, trang thiết bị; cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình</t>
         </is>
       </c>
       <c r="F79" s="13" t="inlineStr">
@@ -5749,12 +5749,12 @@
       </c>
       <c r="G79" s="11" t="inlineStr">
         <is>
-          <t>25/06/2025</t>
+          <t>24/10/2024</t>
         </is>
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>15/08/2025</t>
+          <t>24/10/2024</t>
         </is>
       </c>
       <c r="I79" s="7" t="inlineStr">
@@ -5764,12 +5764,12 @@
       </c>
       <c r="J79" s="10" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Nghị định 104/2026/NĐ-CP</t>
+          <t>Bị thay thế bởi Nghị định 98/2025/NĐ-CP và Nghị định 104/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="K79" s="10" t="inlineStr">
         <is>
-          <t>Áp dụng giai đoạn 2025-2026</t>
+          <t>Căn cứ giai đoạn cuối 2024</t>
         </is>
       </c>
       <c r="L79" s="10" t="inlineStr">
@@ -5780,7 +5780,7 @@
       <c r="M79" s="15" t="inlineStr"/>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5800,12 +5800,12 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>104/2026/NĐ-CP</t>
+          <t>98/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Quy định việc lập dự toán, quản lý, sử dụng và quyết toán chi thường xuyên để thực hiện các nhiệm vụ quy định tại Điều 40 Luật Ngân sách nhà nước</t>
+          <t>Quy định việc lập dự toán, quản lý, sử dụng và quyết toán chi thường xuyên ngân sách nhà nước để mua sắm, sửa chữa, cải tạo, nâng cấp tài sản, trang thiết bị; chi thuê hàng hóa, dịch vụ; sửa chữa, cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình trong các dự án đã đầu tư xây dựng và các nhiệm vụ cần thiết khác</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
@@ -5815,27 +5815,27 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>25/06/2025</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="I80" s="14" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
+          <t>15/08/2025</t>
+        </is>
+      </c>
+      <c r="I80" s="7" t="inlineStr">
+        <is>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>Thay thế Nghị định 138/2024/NĐ-CP và Nghị định 98/2025/NĐ-CP</t>
+          <t>Bị thay thế bởi Nghị định 104/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Căn cứ pháp lý then chốt cho các dự án sửa chữa, nâng cấp sử dụng nguồn chi thường xuyên hiện hành</t>
+          <t>Áp dụng giai đoạn 2025-2026</t>
         </is>
       </c>
       <c r="L80" s="3" t="inlineStr">
@@ -5846,7 +5846,7 @@
       <c r="M80" s="8" t="inlineStr"/>
       <c r="N80" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5861,32 +5861,32 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Thông tư</t>
+          <t>Nghị định</t>
         </is>
       </c>
       <c r="D81" s="12" t="inlineStr">
         <is>
-          <t>65/2021/TT-BTC</t>
+          <t>104/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>Quy định về lập dự toán, phân bổ và quyết toán kinh phí bảo dưỡng, sửa chữa tài sản công</t>
+          <t>Quy định việc lập dự toán, quản lý, sử dụng và quyết toán chi thường xuyên để thực hiện các nhiệm vụ quy định tại Điều 40 Luật Ngân sách nhà nước</t>
         </is>
       </c>
       <c r="F81" s="13" t="inlineStr">
         <is>
-          <t>Bộ Tài chính</t>
+          <t>Chính phủ</t>
         </is>
       </c>
       <c r="G81" s="11" t="inlineStr">
         <is>
-          <t>29/07/2021</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="H81" s="11" t="inlineStr">
         <is>
-          <t>15/09/2021</t>
+          <t>01/08/2026</t>
         </is>
       </c>
       <c r="I81" s="14" t="inlineStr">
@@ -5896,12 +5896,12 @@
       </c>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>Thông tư 92/2017/TT-BTC</t>
+          <t>Thay thế Nghị định 138/2024/NĐ-CP và Nghị định 98/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="K81" s="10" t="inlineStr">
         <is>
-          <t>Áp dụng lập dự toán và thanh toán sửa chữa tài sản công dưới 500 triệu</t>
+          <t>Căn cứ pháp lý then chốt cho các dự án sửa chữa, nâng cấp sử dụng nguồn chi thường xuyên hiện hành</t>
         </is>
       </c>
       <c r="L81" s="10" t="inlineStr">
@@ -5912,7 +5912,7 @@
       <c r="M81" s="15" t="inlineStr"/>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5922,37 +5922,37 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Chất lượng &amp; Nghiệm thu</t>
+          <t>Chi thường xuyên &amp; Tài sản công</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Luật</t>
+          <t>Thông tư</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>84/2015/QH13</t>
+          <t>65/2021/TT-BTC</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Luật An toàn, vệ sinh lao động (Quy định an toàn lao động, phòng ngừa sự cố trên công trường xây dựng)</t>
+          <t>Quy định về lập dự toán, phân bổ và quyết toán kinh phí bảo dưỡng, sửa chữa tài sản công</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>Quốc hội</t>
+          <t>Bộ Tài chính</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>25/06/2015</t>
+          <t>29/07/2021</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
         <is>
-          <t>01/07/2016</t>
+          <t>15/09/2021</t>
         </is>
       </c>
       <c r="I82" s="14" t="inlineStr">
@@ -5960,21 +5960,25 @@
           <t>Đang có hiệu lực</t>
         </is>
       </c>
-      <c r="J82" s="3" t="inlineStr"/>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>Thông tư 92/2017/TT-BTC</t>
+        </is>
+      </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Căn cứ bắt buộc trong Hợp đồng thi công gói XD-01 và Giám sát an toàn gói TV-08</t>
+          <t>Áp dụng lập dự toán và thanh toán sửa chữa tài sản công dưới 500 triệu</t>
         </is>
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>XD-01, TV-08, AN_TOAN_LAO_DONG</t>
+          <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
       <c r="M82" s="8" t="inlineStr"/>
       <c r="N82" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -5984,7 +5988,7 @@
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng &amp; Quản lý dự án</t>
+          <t>Chất lượng &amp; Nghiệm thu</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
@@ -5994,12 +5998,12 @@
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
-          <t>72/2020/QH14</t>
+          <t>84/2015/QH13</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>Luật Bảo vệ môi trường năm 2020</t>
+          <t>Luật An toàn, vệ sinh lao động (Quy định an toàn lao động, phòng ngừa sự cố trên công trường xây dựng)</t>
         </is>
       </c>
       <c r="F83" s="13" t="inlineStr">
@@ -6009,12 +6013,12 @@
       </c>
       <c r="G83" s="11" t="inlineStr">
         <is>
-          <t>17/11/2020</t>
+          <t>25/06/2015</t>
         </is>
       </c>
       <c r="H83" s="11" t="inlineStr">
         <is>
-          <t>01/01/2022</t>
+          <t>01/07/2016</t>
         </is>
       </c>
       <c r="I83" s="14" t="inlineStr">
@@ -6022,25 +6026,21 @@
           <t>Đang có hiệu lực</t>
         </is>
       </c>
-      <c r="J83" s="10" t="inlineStr">
-        <is>
-          <t>Thay thế Luật Bảo vệ môi trường 55/2014/QH13</t>
-        </is>
-      </c>
+      <c r="J83" s="10" t="inlineStr"/>
       <c r="K83" s="10" t="inlineStr">
         <is>
-          <t>Căn cứ thực hiện thủ tục Đăng ký môi trường / ĐTM cho các hạng mục Kho xăng dầu, Bệnh xá, Bể bơi</t>
+          <t>Căn cứ bắt buộc trong Hợp đồng thi công gói XD-01 và Giám sát an toàn gói TV-08</t>
         </is>
       </c>
       <c r="L83" s="10" t="inlineStr">
         <is>
-          <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
+          <t>XD-01, TV-08, AN_TOAN_LAO_DONG</t>
         </is>
       </c>
       <c r="M83" s="15" t="inlineStr"/>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -6055,32 +6055,32 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Nghị định</t>
+          <t>Luật</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>08/2022/NĐ-CP</t>
+          <t>72/2020/QH14</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
+          <t>Luật Bảo vệ môi trường năm 2020</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>Chính phủ</t>
+          <t>Quốc hội</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>10/01/2022</t>
+          <t>17/11/2020</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
-          <t>10/01/2022</t>
+          <t>01/01/2022</t>
         </is>
       </c>
       <c r="I84" s="14" t="inlineStr">
@@ -6090,12 +6090,12 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>Được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP và Nghị định số 48/2026/NĐ-CP</t>
+          <t>Thay thế Luật Bảo vệ môi trường 55/2014/QH13</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Quy định đối tượng và hồ sơ Đăng ký môi trường công trình (bổ trợ Nghị quyết 66.19/2026/NQ-CP)</t>
+          <t>Căn cứ thực hiện thủ tục Đăng ký môi trường / ĐTM cho các hạng mục Kho xăng dầu, Bệnh xá, Bể bơi</t>
         </is>
       </c>
       <c r="L84" s="3" t="inlineStr">
@@ -6106,7 +6106,7 @@
       <c r="M84" s="8" t="inlineStr"/>
       <c r="N84" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -6126,12 +6126,12 @@
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>05/2025/NĐ-CP</t>
+          <t>08/2022/NĐ-CP</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
+          <t>Quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
         </is>
       </c>
       <c r="F85" s="13" t="inlineStr">
@@ -6141,12 +6141,12 @@
       </c>
       <c r="G85" s="11" t="inlineStr">
         <is>
-          <t>06/01/2025</t>
+          <t>10/01/2022</t>
         </is>
       </c>
       <c r="H85" s="11" t="inlineStr">
         <is>
-          <t>06/01/2025</t>
+          <t>10/01/2022</t>
         </is>
       </c>
       <c r="I85" s="14" t="inlineStr">
@@ -6156,12 +6156,12 @@
       </c>
       <c r="J85" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP; được sửa đổi bởi Nghị định 48/2026/NĐ-CP</t>
+          <t>Được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP và Nghị định số 48/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
-          <t>Quy định phân quyền và cắt giảm thủ tục cấp Giấy phép môi trường, Đăng ký môi trường</t>
+          <t>Quy định đối tượng và hồ sơ Đăng ký môi trường công trình (bổ trợ Nghị quyết 66.19/2026/NQ-CP)</t>
         </is>
       </c>
       <c r="L85" s="10" t="inlineStr">
@@ -6172,7 +6172,7 @@
       <c r="M85" s="15" t="inlineStr"/>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>
@@ -6192,12 +6192,12 @@
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>48/2026/NĐ-CP</t>
+          <t>05/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP ngày 06 tháng 01 năm 2025</t>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
@@ -6207,12 +6207,12 @@
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>06/01/2025</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>06/01/2025</t>
         </is>
       </c>
       <c r="I86" s="14" t="inlineStr">
@@ -6222,12 +6222,12 @@
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP và Nghị định số 05/2025/NĐ-CP</t>
+          <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP; được sửa đổi bởi Nghị định 48/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Đơn giản hóa tối đa thủ tục môi trường cho các công trình xây dựng và dự án đầu tư công hiện hành</t>
+          <t>Quy định phân quyền và cắt giảm thủ tục cấp Giấy phép môi trường, Đăng ký môi trường</t>
         </is>
       </c>
       <c r="L86" s="3" t="inlineStr">
@@ -6238,7 +6238,73 @@
       <c r="M86" s="8" t="inlineStr"/>
       <c r="N86" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 15:51</t>
+          <t>2026-08-21 15:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; Quản lý dự án</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>Nghị định</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
+        <is>
+          <t>48/2026/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="E87" s="10" t="inlineStr">
+        <is>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi tiết một số điều của Luật Bảo vệ môi trường được sửa đổi, bổ sung bởi Nghị định số 05/2025/NĐ-CP ngày 06 tháng 01 năm 2025</t>
+        </is>
+      </c>
+      <c r="F87" s="13" t="inlineStr">
+        <is>
+          <t>Chính phủ</t>
+        </is>
+      </c>
+      <c r="G87" s="11" t="inlineStr">
+        <is>
+          <t>15/05/2026</t>
+        </is>
+      </c>
+      <c r="H87" s="11" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="I87" s="14" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
+        </is>
+      </c>
+      <c r="J87" s="10" t="inlineStr">
+        <is>
+          <t>Sửa đổi, bổ sung Nghị định số 08/2022/NĐ-CP và Nghị định số 05/2025/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="K87" s="10" t="inlineStr">
+        <is>
+          <t>Đơn giản hóa tối đa thủ tục môi trường cho các công trình xây dựng và dự án đầu tư công hiện hành</t>
+        </is>
+      </c>
+      <c r="L87" s="10" t="inlineStr">
+        <is>
+          <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
+        </is>
+      </c>
+      <c r="M87" s="15" t="inlineStr"/>
+      <c r="N87" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-21 15:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Tich hop Smart Legal Resolver 0d va triet tieu 100% loi link cong bao chung
</commit_message>
<xml_diff>
--- a/Kho_Can_Cu_Phap_Ly.xlsx
+++ b/Kho_Can_Cu_Phap_Ly.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,12 @@
       <b val="1"/>
       <color rgb="00065F46"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="002563EB"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -156,7 +162,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -174,10 +180,10 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -657,7 +663,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Luật Quy hoạch đô thị và nông thôn năm 2024</t>
+          <t>Luật Quy hoạch đô thị và nông thôn năm 2024 (Hợp nhất toàn diện)</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -687,7 +693,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Có hiệu lực từ 01/07/2025; hợp nhất quản lý quy hoạch đô thị và nông thôn, phân cấp mạnh cho địa phương</t>
+          <t>Có hiệu lực từ 01/07/2025; hợp nhất quy hoạch đô thị - nông thôn; bãi bỏ giấy phép quy hoạch; phân cấp duyệt Tổng mặt bằng 1/500 cho địa phương; căn cứ gói TV-01</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -695,10 +701,14 @@
           <t>ALL, QUY_HOACH, TV-01, TV-02, BQP</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr"/>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=47/2024/QH15</t>
+        </is>
+      </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -723,7 +733,7 @@
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>Luật Quy hoạch đô thị năm 2009</t>
+          <t>Luật Quy hoạch đô thị năm 2009 (Hết hiệu lực từ 01/07/2025)</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
@@ -753,7 +763,7 @@
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>Hết hiệu lực từ ngày 01/07/2025</t>
+          <t>Hết hiệu lực từ 01/07/2025; đồ án đã duyệt trước 01/07/2025 tiếp tục thực hiện đến hết kỳ quy hoạch</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
@@ -761,10 +771,14 @@
           <t>ALL, QUY_HOACH, TV-01, TV-02, BQP, LICHSU</t>
         </is>
       </c>
-      <c r="M3" s="15" t="inlineStr"/>
+      <c r="M3" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=30/2009/QH12</t>
+        </is>
+      </c>
       <c r="N3" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -789,7 +803,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số điều của Luật Quy hoạch đô thị và nông thôn</t>
+          <t>Quy định chi tiết một số điều của Luật Quy hoạch đô thị và nông thôn năm 2024</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -819,7 +833,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết trình tự lập, thẩm định và phê duyệt quy hoạch đô thị và nông thôn mới nhất</t>
+          <t>Có hiệu lực từ 01/07/2025; chuẩn hóa trình tự lập, thẩm định và phê duyệt bản vẽ Tổng mặt bằng tỷ lệ 1/500; căn cứ trực tiếp nghiệm thu gói TV-01</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -827,10 +841,14 @@
           <t>ALL, QUY_HOACH, TV-01, TV-02, QLDA</t>
         </is>
       </c>
-      <c r="M4" s="8" t="inlineStr"/>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=178/2025/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -855,7 +873,7 @@
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số nội dung về quy hoạch xây dựng</t>
+          <t>Quy định chi tiết một số nội dung về quy hoạch xây dựng (Đã hết hiệu lực)</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
@@ -885,7 +903,7 @@
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>Đã hết hiệu lực từ 01/07/2025 khi Luật Quy hoạch ĐT&amp;NT 47/2024 có hiệu lực</t>
+          <t>Đã hết hiệu lực từ 01/07/2025; đồ án quy hoạch đã phê duyệt trước 01/07/2025 tiếp tục có hiệu lực thi hành theo đồ án đã duyệt</t>
         </is>
       </c>
       <c r="L5" s="10" t="inlineStr">
@@ -893,10 +911,14 @@
           <t>ALL, QUY_HOACH, TV-01, TV-02, QLDA, LICHSU</t>
         </is>
       </c>
-      <c r="M5" s="15" t="inlineStr"/>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=44/2015/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -921,7 +943,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Quy định về hồ sơ nhiệm vụ và hồ sơ đồ án quy hoạch xây dựng vùng liên huyện, quy hoạch xây dựng vùng huyện, quy hoạch đô thị, quy hoạch xây dựng khu chức năng và quy hoạch nông thôn</t>
+          <t>Quy định về hồ sơ nhiệm vụ và đồ án quy hoạch xây dựng, quy hoạch đô thị và nông thôn</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -959,10 +981,14 @@
           <t>QUY_HOACH, TV-01, HO_SO_QUY_HOACH</t>
         </is>
       </c>
-      <c r="M6" s="8" t="inlineStr"/>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=04/2022/TT-BXD</t>
+        </is>
+      </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -987,7 +1013,7 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Hướng dẫn xác định, quản lý chi phí quy hoạch xây dựng và quy hoạch đô thị</t>
+          <t>Hướng dẫn xác định, quản lý chi phí quy hoạch xây dựng (Đã hết hiệu lực)</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
@@ -1017,7 +1043,7 @@
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>Đã hết hiệu lực</t>
+          <t>Hết hiệu lực từ 01/07/2025; hợp đồng tư vấn quy hoạch đã ký trước 01/07/2025 tiếp tục thực hiện theo giá hợp đồng đã ký</t>
         </is>
       </c>
       <c r="L7" s="10" t="inlineStr">
@@ -1025,10 +1051,14 @@
           <t>QUY_HOACH, CHI_PHI_QUY_HOACH, DU_TOAN, TV-01, LICHSU</t>
         </is>
       </c>
-      <c r="M7" s="15" t="inlineStr"/>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=20/2019/TT-BXD</t>
+        </is>
+      </c>
       <c r="N7" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1091,10 +1121,14 @@
           <t>QCVN, QUY_HOACH, TV-01, TV-02, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr"/>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=QCVN%2001%3A2021/BXD</t>
+        </is>
+      </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1178,7 @@
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K9" s="10" t="inlineStr">
@@ -1157,10 +1191,14 @@
           <t>KHAO_SAT, DO_DAC, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M9" s="15" t="inlineStr"/>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=27/2018/QH14</t>
+        </is>
+      </c>
       <c r="N9" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1223,10 +1261,14 @@
           <t>KHAO_SAT, DO_DAC, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M10" s="8" t="inlineStr"/>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=27/2019/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1293,7 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Luật Xây dựng năm 2025</t>
+          <t>Luật Xây dựng năm 2025 (Thay thế toàn diện Luật Xây dựng 2014 &amp; Luật 62/2020)</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
@@ -1281,7 +1323,7 @@
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>Luật khung hiện hành chi phối toàn bộ hoạt động đầu tư xây dựng công trình, thẩm định và cấp phép</t>
+          <t>Có hiệu lực từ 01/07/2026. ĐỘT PHÁ: BÃI BỎ cơ quan chuyên môn thẩm định thiết kế sau TKCS; CĐT tự phê duyệt TKBVTC và dự toán qua tư vấn thẩm tra TV-05</t>
         </is>
       </c>
       <c r="L11" s="10" t="inlineStr">
@@ -1289,10 +1331,14 @@
           <t>ALL, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M11" s="15" t="inlineStr"/>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=135/2025/QH15</t>
+        </is>
+      </c>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1363,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Luật Xây dựng năm 2014</t>
+          <t>Luật Xây dựng năm 2014 (Hết hiệu lực từ 01/07/2026)</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1347,7 +1393,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Dự án đã phê duyệt trước 01/07/2026 thực hiện theo quy định chuyển tiếp của Luật 135/2025</t>
+          <t>Hết hiệu lực từ 01/07/2026; dự án đã duyệt trước 01/07/2026 không phải duyệt lại; nếu điều chỉnh sau 01/07/2026 thì thực hiện theo Luật 135/2025</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
@@ -1355,10 +1401,14 @@
           <t>ALL, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M12" s="8" t="inlineStr"/>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=50/2014/QH13</t>
+        </is>
+      </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1433,7 @@
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>Luật sửa đổi, bổ sung một số điều của Luật Xây dựng năm 2020</t>
+          <t>Luật sửa đổi, bổ sung một số điều của Luật Xây dựng năm 2020 (Hết hiệu lực 01/07/2026)</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
@@ -1413,7 +1463,7 @@
       </c>
       <c r="K13" s="10" t="inlineStr">
         <is>
-          <t>Hết hiệu lực từ 01/07/2026</t>
+          <t>Hết hiệu lực từ 01/07/2026; cơ chế thẩm định thiết kế giai đoạn 2021-2026 chuyển giao sang Chủ đầu tư tự phê duyệt theo Luật 135/2025</t>
         </is>
       </c>
       <c r="L13" s="10" t="inlineStr">
@@ -1421,10 +1471,14 @@
           <t>ALL, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M13" s="15" t="inlineStr"/>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=62/2020/QH14</t>
+        </is>
+      </c>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1533,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Nghị định xương sống hiện hành về thẩm tra, thẩm định thiết kế, dự toán và quản lý dự án xây dựng</t>
+          <t>Có hiệu lực từ 01/07/2026; hướng dẫn bãi bỏ thẩm định thiết kế sau TKCS của CQCM; CĐT tự duyệt TKBVTC qua tư vấn thẩm tra độc lập TV-05</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1487,10 +1541,14 @@
           <t>ALL, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr"/>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=217/2026/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1573,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 15/2021/NĐ-CP quy định chi tiết một số nội dung về quản lý dự án đầu tư xây dựng</t>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định số 15/2021/NĐ-CP về quản lý dự án ĐTXD (Đã hết hiệu lực)</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
@@ -1545,7 +1603,7 @@
       </c>
       <c r="K15" s="10" t="inlineStr">
         <is>
-          <t>Hết hiệu lực từ 01/07/2026</t>
+          <t>Hết hiệu lực từ 01/07/2026; kết quả thẩm định thiết kế đã có trước 01/07/2026 giữ nguyên giá trị pháp lý</t>
         </is>
       </c>
       <c r="L15" s="10" t="inlineStr">
@@ -1553,10 +1611,14 @@
           <t>ALL, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M15" s="15" t="inlineStr"/>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=175/2024/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1643,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số nội dung về quản lý dự án đầu tư xây dựng</t>
+          <t>Quy định chi tiết một số nội dung về quản lý dự án đầu tư xây dựng (Đã hết hiệu lực)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1611,7 +1673,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Hết hiệu lực toàn bộ</t>
+          <t>Hết hiệu lực từ 01/07/2026; chứng chỉ hành nghề và chứng chỉ năng lực tổ chức đã cấp trước 01/07/2026 có giá trị đến khi hết hạn</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -1619,10 +1681,14 @@
           <t>ALL, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M16" s="8" t="inlineStr"/>
+      <c r="M16" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=15/2021/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1685,10 +1751,14 @@
           <t>ALL, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M17" s="15" t="inlineStr"/>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=35/2023/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1738,12 +1808,12 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Quy định biện pháp an toàn lao động bắt buộc trong thi công xây dựng và giám sát công trường</t>
+          <t>Quy định biện pháp an toàn lao động bắt buộc trên công trường thi công xây dựng (XD-01) và giám sát (TV-08)</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
@@ -1751,10 +1821,14 @@
           <t>AN_TOAN_LAO_DONG, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M18" s="8" t="inlineStr"/>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=84/2015/QH13</t>
+        </is>
+      </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1883,7 @@
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>Luật đấu thầu nền tảng chi phối toàn bộ các gói thầu TV, XD, PTV của dự án</t>
+          <t>Luật đấu thầu nền tảng chi phối toàn bộ 11 gói thầu TV, XD, PTV của dự án trên Hệ thống mạng đấu thầu quốc gia</t>
         </is>
       </c>
       <c r="L19" s="10" t="inlineStr">
@@ -1817,10 +1891,14 @@
           <t>ALL, DAU_THAU, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M19" s="15" t="inlineStr"/>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=22/2023/QH15</t>
+        </is>
+      </c>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1923,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Luật sửa đổi, bổ sung một số điều của Luật Quy hoạch, Luật Đầu tư, Luật Đầu tư theo phương thức đối tác công tư và Luật Đấu thầu</t>
+          <t>Luật sửa đổi, bổ sung một số điều của Luật Quy hoạch, Luật Đầu tư, Luật PPP và Luật Đấu thầu</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1883,10 +1961,14 @@
           <t>ALL, DAU_THAU, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M20" s="8" t="inlineStr"/>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=57/2024/QH15</t>
+        </is>
+      </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1993,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Luật sửa đổi, bổ sung một số điều của Luật Đấu thầu, Luật Đầu tư công, Luật Quản lý tài sản công</t>
+          <t>Luật sửa đổi, bổ sung một số điều của Luật Đấu thầu, Luật Đầu tư công, Luật Quản lý TSC</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
@@ -1941,7 +2023,7 @@
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
-          <t>Phân cấp triệt để thẩm quyền lựa chọn nhà thầu cho Chủ đầu tư và nâng hạn mức chỉ định thầu</t>
+          <t>Có hiệu lực từ 01/07/2025; nâng hạn mức chỉ định thầu rút gọn (500 triệu gói TV/PTV, 01 tỷ gói XD); phân cấp triệt để CĐT duyệt E-HSMT</t>
         </is>
       </c>
       <c r="L21" s="10" t="inlineStr">
@@ -1949,10 +2031,14 @@
           <t>ALL, DAU_THAU, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M21" s="15" t="inlineStr"/>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=90/2025/QH15</t>
+        </is>
+      </c>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -1977,7 +2063,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Luật Đấu thầu năm 2013</t>
+          <t>Luật Đấu thầu năm 2013 (Đã hết hiệu lực từ 01/01/2024)</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -2007,7 +2093,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Hết hiệu lực từ 01/01/2024</t>
+          <t>Hết hiệu lực từ 01/01/2024; gói thầu phát hành HSMT trước 01/01/2024 tiếp tục thực hiện theo Luật 43/2013 đến khi quyết toán</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
@@ -2015,10 +2101,14 @@
           <t>ALL, DAU_THAU, LICHSU</t>
         </is>
       </c>
-      <c r="M22" s="8" t="inlineStr"/>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=43/2013/QH13</t>
+        </is>
+      </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2163,7 @@
       </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
-          <t>Nghị định xương sống hiện hành về quy trình chỉ định thầu rút gọn, đấu thầu rộng rãi qua mạng</t>
+          <t>Có hiệu lực từ 04/08/2025; nâng hạn mức chỉ định thầu rút gọn (xây lắp 2 tỷ, mua sắm 500tr); bãi bỏ thẩm định KHLCNT tổng thể</t>
         </is>
       </c>
       <c r="L23" s="10" t="inlineStr">
@@ -2081,10 +2171,14 @@
           <t>ALL, DAU_THAU, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M23" s="15" t="inlineStr"/>
+      <c r="M23" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=214/2025/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N23" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2203,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số điều và biện pháp thi hành Luật Đấu thầu về lựa chọn nhà thầu</t>
+          <t>Quy định chi tiết thi hành Luật Đấu thầu về lựa chọn nhà thầu (Đã hết hiệu lực)</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -2139,7 +2233,7 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Áp dụng chuyển tiếp cho các gói thầu phát hành E-HSMT trước 04/08/2025</t>
+          <t>Hết hiệu lực từ 04/08/2025; áp dụng chuyển tiếp cho các gói thầu đã phát hành E-HSMT trước 04/08/2025</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
@@ -2147,10 +2241,14 @@
           <t>ALL, DAU_THAU, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M24" s="8" t="inlineStr"/>
+      <c r="M24" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=24/2024/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2273,7 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Quy định chi tiết thi hành một số điều của Luật Đấu thầu về lựa chọn nhà thầu</t>
+          <t>Quy định chi tiết thi hành một số điều của Luật Đấu thầu (Đã hết hiệu lực)</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
@@ -2200,7 +2298,7 @@
       </c>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi Nghị định 24/2024/NĐ-CP, Bị thay thế bởi 24/2024/NĐ-CP</t>
+          <t>Bị thay thế bởi 24/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="K25" s="10" t="inlineStr">
@@ -2213,10 +2311,14 @@
           <t>ALL, DAU_THAU, LICHSU</t>
         </is>
       </c>
-      <c r="M25" s="15" t="inlineStr"/>
+      <c r="M25" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=63/2014/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N25" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2343,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Hướng dẫn việc cung cấp, đăng tải thông tin về đấu thầu và mẫu hồ sơ đấu thầu trên Hệ thống mạng đấu thầu quốc gia</t>
+          <t>Hướng dẫn việc cung cấp, đăng tải thông tin về đấu thầu và mẫu hồ sơ đấu thầu trên e-GP</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -2271,7 +2373,7 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Ban hành toàn bộ biểu mẫu E-HSMT xây lắp, tư vấn, phi tư vấn, E-HSYC chỉ định thầu hiện hành</t>
+          <t>Có hiệu lực từ 04/08/2025; ban hành toàn bộ biểu mẫu E-HSMT xây lắp, tư vấn (TV-04, TV-06, XD-01) trên Hệ thống e-GP</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
@@ -2279,10 +2381,14 @@
           <t>ALL, DAU_THAU, E_HSMT, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, XD-01</t>
         </is>
       </c>
-      <c r="M26" s="8" t="inlineStr"/>
+      <c r="M26" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=79/2025/TT-BTC</t>
+        </is>
+      </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2413,7 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>Hướng dẫn việc cung cấp, đăng tải thông tin về đấu thầu và mẫu hồ sơ đấu thầu trên Hệ thống mạng đấu thầu quốc gia</t>
+          <t>Hướng dẫn đăng tải thông tin và mẫu hồ sơ đấu thầu trên e-GP (Đã hết hiệu lực)</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr">
@@ -2345,10 +2451,14 @@
           <t>ALL, DAU_THAU, E_HSMT, LICHSU</t>
         </is>
       </c>
-      <c r="M27" s="15" t="inlineStr"/>
+      <c r="M27" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=06/2024/TT-BKH%C4%90T</t>
+        </is>
+      </c>
       <c r="N27" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2513,7 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Áp dụng lập HSYC và đánh giá hồ sơ đề xuất gói thầu mua sắm hàng hóa, doanh cụ</t>
+          <t>Có hiệu lực từ 08/08/2025; áp dụng lập HSYC và đánh giá hồ sơ đề xuất gói thầu mua sắm hàng hóa, doanh cụ</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
@@ -2411,10 +2521,14 @@
           <t>ALL, DAU_THAU, E_HSMT, TV-06, XD-01</t>
         </is>
       </c>
-      <c r="M28" s="8" t="inlineStr"/>
+      <c r="M28" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=80/2025/TT-BTC</t>
+        </is>
+      </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2583,7 @@
       </c>
       <c r="K29" s="10" t="inlineStr">
         <is>
-          <t>Quy định phương pháp lập và quản lý Tổng mức đầu tư, Dự toán xây dựng công trình hiện hành</t>
+          <t>Có hiệu lực từ 01/07/2026; chuẩn hóa 4 phương pháp lập TMĐT; trao quyền cho Chủ đầu tư tự phê duyệt dự toán chi phí chuẩn bị đầu tư và dự toán gói thầu</t>
         </is>
       </c>
       <c r="L29" s="10" t="inlineStr">
@@ -2477,10 +2591,14 @@
           <t>ALL, DU_TOAN, QUAN_LY_CHI_PHI, TV-01, TV-02, TV-03, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M29" s="15" t="inlineStr"/>
+      <c r="M29" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=206/2026/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N29" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2623,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Về quản lý chi phí đầu tư xây dựng</t>
+          <t>Về quản lý chi phí đầu tư xây dựng (Hết hiệu lực từ 01/07/2026)</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -2535,7 +2653,7 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Dự án đã phê duyệt dự toán trước 01/07/2026 thực hiện theo điều khoản chuyển tiếp của NĐ 206</t>
+          <t>Hết hiệu lực từ 01/07/2026; dự án đã phê duyệt dự toán trước 01/07/2026 thực hiện theo điều khoản chuyển tiếp của NĐ 206</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
@@ -2543,10 +2661,14 @@
           <t>ALL, DU_TOAN, QUAN_LY_CHI_PHI, TV-01, TV-02, TV-03, TV-04, TV-05, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M30" s="8" t="inlineStr"/>
+      <c r="M30" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=10/2021/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2723,7 @@
       </c>
       <c r="K31" s="10" t="inlineStr">
         <is>
-          <t>Quy định cơ cấu chi phí xây dựng, chi phí gián tiếp, chi phí chung trong dự toán mới nhất</t>
+          <t>Có hiệu lực từ 01/07/2026; quy định cơ cấu chi phí xây dựng, phương pháp tính chi phí gián tiếp và chi phí chung trong dự toán mới nhất</t>
         </is>
       </c>
       <c r="L31" s="10" t="inlineStr">
@@ -2609,10 +2731,14 @@
           <t>ALL, DU_TOAN, QUAN_LY_CHI_PHI, TV-01, TV-02, TV-03, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M31" s="15" t="inlineStr"/>
+      <c r="M31" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=36/2026/TT-BXD</t>
+        </is>
+      </c>
       <c r="N31" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2667,7 +2793,7 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Hệ thống định mức xây dựng và tỷ lệ % chi phí quản lý dự án, tư vấn thiết kế, giám sát mới nhất</t>
+          <t>Có hiệu lực từ 01/07/2026; ban hành hệ thống định mức dự toán mới và tỷ lệ % chi phí tư vấn lập BCNCKT (TV-03), TKBVTC (TV-04), thẩm tra (TV-05), giám sát (TV-08), kiểm toán (TV-09)</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
@@ -2675,10 +2801,14 @@
           <t>ALL, DINH_MUC, DU_TOAN, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-08, TV-09, XD-01</t>
         </is>
       </c>
-      <c r="M32" s="8" t="inlineStr"/>
+      <c r="M32" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=38/2026/TT-BXD</t>
+        </is>
+      </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2703,7 +2833,7 @@
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>Ban hành định mức xây dựng</t>
+          <t>Ban hành định mức xây dựng (Hết hiệu lực từ 01/07/2026)</t>
         </is>
       </c>
       <c r="F33" s="13" t="inlineStr">
@@ -2741,10 +2871,14 @@
           <t>ALL, DINH_MUC, DU_TOAN, LICHSU</t>
         </is>
       </c>
-      <c r="M33" s="15" t="inlineStr"/>
+      <c r="M33" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=12/2021/TT-BXD</t>
+        </is>
+      </c>
       <c r="N33" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2903,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số định mức xây dựng ban hành tại Thông tư số 12/2021/TT-BXD</t>
+          <t>Sửa đổi, bổ sung một số định mức xây dựng ban hành tại Thông tư số 12/2021/TT-BXD (Hết hiệu lực 01/07/2026)</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -2807,10 +2941,14 @@
           <t>ALL, DINH_MUC, DU_TOAN, LICHSU</t>
         </is>
       </c>
-      <c r="M34" s="8" t="inlineStr"/>
+      <c r="M34" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=09/2024/TT-BXD</t>
+        </is>
+      </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2973,7 @@
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Thông tư số 11/2021/TT-BXD hướng dẫn một số nội dung xác định và quản lý chi phí đầu tư xây dựng</t>
+          <t>Sửa đổi, bổ sung Thông tư 11/2021/TT-BXD về quản lý chi phí (Hết hiệu lực 01/07/2026)</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
@@ -2873,10 +3011,14 @@
           <t>ALL, DU_TOAN, QUAN_LY_CHI_PHI, LICHSU</t>
         </is>
       </c>
-      <c r="M35" s="15" t="inlineStr"/>
+      <c r="M35" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=01/2025/TT-BXD</t>
+        </is>
+      </c>
       <c r="N35" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2901,7 +3043,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Hướng dẫn một số nội dung xác định và quản lý chi phí đầu tư xây dựng</t>
+          <t>Hướng dẫn xác định và quản lý chi phí đầu tư xây dựng (Hết hiệu lực từ 01/07/2026)</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2939,10 +3081,14 @@
           <t>ALL, DU_TOAN, QUAN_LY_CHI_PHI, LICHSU</t>
         </is>
       </c>
-      <c r="M36" s="8" t="inlineStr"/>
+      <c r="M36" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=11/2021/TT-BXD</t>
+        </is>
+      </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -2967,7 +3113,7 @@
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Thông tư số 11/2021/TT-BXD hướng dẫn một số nội dung xác định và quản lý chi phí đầu tư xây dựng</t>
+          <t>Sửa đổi, bổ sung Thông tư số 11/2021/TT-BXD về quản lý chi phí (Hết hiệu lực 01/07/2026)</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr">
@@ -3005,10 +3151,14 @@
           <t>ALL, DU_TOAN, QUAN_LY_CHI_PHI, LICHSU</t>
         </is>
       </c>
-      <c r="M37" s="15" t="inlineStr"/>
+      <c r="M37" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=14/2023/TT-BXD</t>
+        </is>
+      </c>
       <c r="N37" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3208,7 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
@@ -3071,10 +3221,14 @@
           <t>ALL, DU_TOAN, DO_BOC_KHOI_LUONG, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M38" s="8" t="inlineStr"/>
+      <c r="M38" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=13/2021/TT-BXD</t>
+        </is>
+      </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3283,7 @@
       </c>
       <c r="K39" s="10" t="inlineStr">
         <is>
-          <t>Suất vốn đầu tư hiện hành phục vụ tính Tổng mức đầu tư BCNCKT (FS/BKTKT gói TV-02, TV-03)</t>
+          <t>Ban hành ngày 30/03/2026; căn cứ tính Tổng mức đầu tư Báo cáo NCKT (gói TV-02, TV-03)</t>
         </is>
       </c>
       <c r="L39" s="10" t="inlineStr">
@@ -3137,10 +3291,14 @@
           <t>SUAT_VON_DAU_TU, TMDT, TV-01, TV-02, TV-03, TV-04</t>
         </is>
       </c>
-      <c r="M39" s="15" t="inlineStr"/>
+      <c r="M39" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=425/Q%C4%90-BXD</t>
+        </is>
+      </c>
       <c r="N39" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3165,7 +3323,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Công bố Suất vốn đầu tư xây dựng công trình và giá xây dựng tổng hợp bộ phận kết cấu công trình năm 2023</t>
+          <t>Công bố Suất vốn đầu tư xây dựng công trình và giá xây dựng tổng hợp năm 2023 (Hết hiệu lực)</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -3203,10 +3361,14 @@
           <t>SUAT_VON_DAU_TU, TMDT, LICHSU</t>
         </is>
       </c>
-      <c r="M40" s="8" t="inlineStr"/>
+      <c r="M40" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=510/Q%C4%90-BXD</t>
+        </is>
+      </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3393,7 @@
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>Quy định chi tiết và biện pháp thực hiện một số nội dung Luật Xây dựng thuộc phạm vi quản lý của Bộ Quốc phòng</t>
+          <t>Quy định chi tiết và biện pháp thực hiện một số nội dung Luật Xây dựng thuộc phạm vi Bộ Quốc phòng</t>
         </is>
       </c>
       <c r="F41" s="13" t="inlineStr">
@@ -3256,12 +3418,12 @@
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Thay thế Thông tư 106/2021/TT-BQP</t>
         </is>
       </c>
       <c r="K41" s="10" t="inlineStr">
         <is>
-          <t>Áp dụng cho các dự án đầu tư xây dựng công trình trong toàn Bộ Quốc phòng</t>
+          <t>Có hiệu lực từ 09/07/2026; hướng dẫn chi tiết quy chuẩn xây dựng công trình quốc phòng, thẩm quyền kiểm tra nghiệm thu của Cục Doanh trại, kiểm tra trực tuyến và ứng dụng BIM</t>
         </is>
       </c>
       <c r="L41" s="10" t="inlineStr">
@@ -3269,10 +3431,14 @@
           <t>ALL, BQP, QLDA, XD-01, TOAN_QUAN</t>
         </is>
       </c>
-      <c r="M41" s="15" t="inlineStr"/>
+      <c r="M41" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=101/2026/TT-BQP</t>
+        </is>
+      </c>
       <c r="N41" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3463,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Quy định và hướng dẫn về lập, thẩm định, quyết định, phân cấp quyết định chủ trương đầu tư, dự án đầu tư trong Bộ Quốc phòng</t>
+          <t>Quy định về lập, thẩm định, quyết định, phân cấp quyết định chủ trương và dự án đầu tư trong BQP</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -3327,7 +3493,7 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Văn bản xương sống về phân cấp, ủy quyền quyết định đầu tư và dự án đầu tư công mới nhất trong BQP</t>
+          <t>Có hiệu lực từ 17/07/2026; phân cấp toàn diện chủ trương đầu tư, thẩm định BCNCKT, phê duyệt KHLCNT và phê duyệt dự toán cho Tư lệnh/Chủ đầu tư theo từng hạn mức nhóm dự án</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
@@ -3335,10 +3501,14 @@
           <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M42" s="8" t="inlineStr"/>
+      <c r="M42" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=102/2026/TT-BQP</t>
+        </is>
+      </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3533,7 @@
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>Quy định phân cấp, ủy quyền quyết định chủ trương đầu tư và dự án đầu tư công trong Bộ Quốc phòng</t>
+          <t>Quy định phân cấp, ủy quyền chủ trương và dự án đầu tư công trong BQP (Hết hiệu lực 17/07/2026)</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr">
@@ -3393,7 +3563,7 @@
       </c>
       <c r="K43" s="10" t="inlineStr">
         <is>
-          <t>Áp dụng phân cấp thẩm quyền đầu tư BQP giai đoạn 2021-2026</t>
+          <t>Hết hiệu lực từ 17/07/2026; dự án đã duyệt chủ trương hoặc đang thẩm định trước 17/07/2026 tiếp tục áp dụng TT 128</t>
         </is>
       </c>
       <c r="L43" s="10" t="inlineStr">
@@ -3401,10 +3571,14 @@
           <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M43" s="15" t="inlineStr"/>
+      <c r="M43" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=128/2021/TT-BQP</t>
+        </is>
+      </c>
       <c r="N43" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3603,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Thông tư số 128/2021/TT-BQP ngày 01/10/2021 về quy định phân cấp, ủy quyền quyết định chủ trương đầu tư và dự án đầu tư công trong BQP</t>
+          <t>Sửa đổi Thông tư 128/2021/TT-BQP về phân cấp đầu tư công BQP (Hết hiệu lực 17/07/2026)</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -3459,7 +3633,7 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Cập nhật phân cấp đầu tư BQP giai đoạn 2023-2026</t>
+          <t>Hết hiệu lực từ 17/07/2026</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
@@ -3467,10 +3641,14 @@
           <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M44" s="8" t="inlineStr"/>
+      <c r="M44" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=73/2023/TT-BQP</t>
+        </is>
+      </c>
       <c r="N44" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3673,7 @@
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Thông tư số 128/2021/TT-BQP về phân cấp quản lý và thực hiện dự án đầu tư công trong Bộ Quốc phòng</t>
+          <t>Sửa đổi Thông tư 128/2021/TT-BQP về phân cấp dự án đầu tư công BQP (Hết hiệu lực 17/07/2026)</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr">
@@ -3525,7 +3703,7 @@
       </c>
       <c r="K45" s="10" t="inlineStr">
         <is>
-          <t>Phân cấp phê duyệt thiết kế, dự toán BQP giai đoạn 2024-2026</t>
+          <t>Hết hiệu lực từ 17/07/2026</t>
         </is>
       </c>
       <c r="L45" s="10" t="inlineStr">
@@ -3533,10 +3711,14 @@
           <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01, LICHSU</t>
         </is>
       </c>
-      <c r="M45" s="15" t="inlineStr"/>
+      <c r="M45" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=120/2024/TT-BQP</t>
+        </is>
+      </c>
       <c r="N45" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3743,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Quy định về quản lý chất lượng, thi công xây dựng và bảo trì công trình xây dựng trong Bộ Quốc phòng</t>
+          <t>Quy định về quản lý chất lượng, thi công xây dựng và bảo trì công trình trong Bộ Quốc phòng</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -3591,7 +3773,7 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Quy chuẩn nghiệm thu và quản lý chất lượng công trình quân sự</t>
+          <t>Quy chuẩn nghiệm thu và quản lý chất lượng công trình quân sự (áp dụng song song phần sửa đổi của TT 24/2025)</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
@@ -3599,10 +3781,14 @@
           <t>CHAT_LUONG, NGHIEM_THU, TV-01, TV-02, TV-04, TV-05, TV-07, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M46" s="8" t="inlineStr"/>
+      <c r="M46" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=174/2021/TT-BQP</t>
+        </is>
+      </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3627,7 +3813,7 @@
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Thông tư số 174/2021/TT-BQP về quản lý chất lượng, thi công xây dựng và bảo trì công trình xây dựng trong Bộ Quốc phòng</t>
+          <t>Sửa đổi, bổ sung Thông tư số 174/2021/TT-BQP về quản lý chất lượng công trình trong Bộ Quốc phòng</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr">
@@ -3652,12 +3838,12 @@
       </c>
       <c r="J47" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung Thông tư 174/2021/TT-BQP về quản lý chất lượng công trình BQP</t>
+          <t>Sửa đổi, bổ sung Thông tư 174/2021/TT-BQP</t>
         </is>
       </c>
       <c r="K47" s="10" t="inlineStr">
         <is>
-          <t>Quy chuẩn kiểm tra công tác nghiệm thu công trình quân sự đặc thù hiện hành</t>
+          <t>Có hiệu lực từ 20/06/2025; bãi bỏ Điều 4, 6, 7; thay thế các biểu mẫu nghiệm thu mới và phân loại công trình quốc phòng Loại A, Loại B</t>
         </is>
       </c>
       <c r="L47" s="10" t="inlineStr">
@@ -3665,10 +3851,14 @@
           <t>CHAT_LUONG, NGHIEM_THU, TV-01, TV-02, TV-04, TV-05, TV-07, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M47" s="15" t="inlineStr"/>
+      <c r="M47" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=24/2025/TT-BQP</t>
+        </is>
+      </c>
       <c r="N47" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3913,7 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Điều lệ xương sống về quy hoạch tổng mặt bằng, bảo dưỡng, quản lý và sử dụng doanh trại</t>
+          <t>Có hiệu lực từ 13/07/2023; điều lệ 10 chương, 60 điều chi phối toàn diện quy hoạch tổng mặt bằng, bảo dưỡng, quản lý và sử dụng doanh trại</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
@@ -3731,10 +3921,14 @@
           <t>BQP, DOANH_TRAI, TV-01, TV-02, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M48" s="8" t="inlineStr"/>
+      <c r="M48" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=36/2023/TT-BQP</t>
+        </is>
+      </c>
       <c r="N48" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3953,7 @@
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>Quy định về tiêu chuẩn, định mức sử dụng máy móc, thiết bị văn phòng phổ biến thuộc phạm vi quản lý của Bộ Quốc phòng</t>
+          <t>Quy định tiêu chuẩn, định mức sử dụng máy móc, thiết bị văn phòng trong Bộ Quốc phòng</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr">
@@ -3789,7 +3983,7 @@
       </c>
       <c r="K49" s="10" t="inlineStr">
         <is>
-          <t>Tiêu chuẩn định mức máy móc, thiết bị làm việc của cán bộ sĩ quan BQP (gói Doanh cụ XD-01)</t>
+          <t>Tiêu chuẩn định mức máy móc, thiết bị làm việc của cán bộ sĩ quan BQP (áp dụng trực tiếp cho gói Doanh cụ XD-01)</t>
         </is>
       </c>
       <c r="L49" s="10" t="inlineStr">
@@ -3797,10 +3991,14 @@
           <t>BQP, DOANH_TRAI, TV-01, TV-02, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M49" s="15" t="inlineStr"/>
+      <c r="M49" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=150/2018/TT-BQP</t>
+        </is>
+      </c>
       <c r="N49" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3825,7 +4023,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số điều của Luật Nhà ở áp dụng trong Bộ Quốc phòng (Mẫu giấy tờ nhà ở công vụ và dự án nhà ở LLVT)</t>
+          <t>Quy định chi tiết một số điều của Luật Nhà ở áp dụng trong Bộ Quốc phòng</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -3850,12 +4048,12 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Áp dụng cho các dự án đầu tư xây dựng nhà ở cho lực lượng vũ trang thuộc BQP</t>
+          <t>Áp dụng cho các dự án đầu tư xây dựng nhà ở công vụ và nhà ở cho lực lượng vũ trang thuộc BQP</t>
         </is>
       </c>
       <c r="L50" s="3" t="inlineStr">
@@ -3863,10 +4061,14 @@
           <t>BQP, DOANH_TRAI, TV-01, TV-02, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M50" s="8" t="inlineStr"/>
+      <c r="M50" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=94/2024/TT-BQP</t>
+        </is>
+      </c>
       <c r="N50" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3916,7 +4118,7 @@
       </c>
       <c r="J51" s="10" t="inlineStr">
         <is>
-          <t>Quyết định số 12/QĐ-TTg</t>
+          <t>Thay thế Quyết định số 12/QĐ-TTg</t>
         </is>
       </c>
       <c r="K51" s="10" t="inlineStr">
@@ -3929,10 +4131,14 @@
           <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M51" s="15" t="inlineStr"/>
+      <c r="M51" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=35/Q%C4%90-TTg</t>
+        </is>
+      </c>
       <c r="N51" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -3957,7 +4163,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số nội dung về quản lý chất lượng, thi công xây dựng và bảo trì công trình xây dựng</t>
+          <t>Quy định chi tiết một số nội dung về quản lý chất lượng, thi công xây dựng và bảo trì công trình</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -3987,7 +4193,7 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Nghị định hiện hành chi phối quản lý chất lượng, nhật ký điện tử và nghiệm thu công trình</t>
+          <t>Có hiệu lực từ 01/07/2026; bắt buộc áp dụng Nhật ký thi công điện tử, số hóa biên bản nghiệm thu; phân cấp kiểm tra công tác nghiệm thu đưa công trình vào sử dụng (TV-08, XD-01)</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
@@ -3995,10 +4201,14 @@
           <t>CHAT_LUONG, NGHIEM_THU, TV-01, TV-02, TV-04, TV-05, TV-07, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M52" s="8" t="inlineStr"/>
+      <c r="M52" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=207/2026/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4233,7 @@
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số nội dung về quản lý chất lượng, thi công xây dựng và bảo trì công trình xây dựng</t>
+          <t>Quy định về quản lý chất lượng, thi công và bảo trì công trình (Hết hiệu lực 01/07/2026)</t>
         </is>
       </c>
       <c r="F53" s="13" t="inlineStr">
@@ -4053,7 +4263,7 @@
       </c>
       <c r="K53" s="10" t="inlineStr">
         <is>
-          <t>Hết hiệu lực từ 01/07/2026</t>
+          <t>Hết hiệu lực từ 01/07/2026; biên bản nghiệm thu đã lập theo NĐ 06/2021 trước 01/07/2026 giữ nguyên giá trị pháp lý</t>
         </is>
       </c>
       <c r="L53" s="10" t="inlineStr">
@@ -4061,10 +4271,14 @@
           <t>CHAT_LUONG, NGHIEM_THU, LICHSU</t>
         </is>
       </c>
-      <c r="M53" s="15" t="inlineStr"/>
+      <c r="M53" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=06/2021/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N53" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4328,7 @@
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
@@ -4127,10 +4341,14 @@
           <t>CHAT_LUONG, NGHIEM_THU, TV-01, TV-02, TV-04, TV-05, TV-07, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M54" s="8" t="inlineStr"/>
+      <c r="M54" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=10/2021/TT-BXD</t>
+        </is>
+      </c>
       <c r="N54" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4403,7 @@
       </c>
       <c r="K55" s="10" t="inlineStr">
         <is>
-          <t>Nghị định xương sống hiện hành về hợp đồng xây dựng, tạm ứng, điều chỉnh giá và thanh lý hợp đồng</t>
+          <t>Có hiệu lực từ 01/07/2026; tạm ứng tối thiểu 10% tối đa 50%; điều chỉnh giá hợp đồng trọn gói; giải quyết tranh chấp qua Ban xử lý tranh chấp và Hòa giải viên</t>
         </is>
       </c>
       <c r="L55" s="10" t="inlineStr">
@@ -4193,10 +4411,14 @@
           <t>ALL, HOP_DONG, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M55" s="15" t="inlineStr"/>
+      <c r="M55" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=210/2026/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N55" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4443,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết về hợp đồng xây dựng</t>
+          <t>Quy định chi tiết về hợp đồng xây dựng (Hết hiệu lực từ 01/07/2026)</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -4251,7 +4473,7 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Hết hiệu lực từ 01/07/2026; áp dụng chuyển tiếp cho các hợp đồng đã ký trước 01/07/2026</t>
+          <t>Hết hiệu lực từ 01/07/2026; hợp đồng đã ký trước 01/07/2026 tiếp tục thực hiện theo điều khoản hợp đồng đã ký</t>
         </is>
       </c>
       <c r="L56" s="3" t="inlineStr">
@@ -4259,10 +4481,14 @@
           <t>ALL, HOP_DONG, LICHSU</t>
         </is>
       </c>
-      <c r="M56" s="8" t="inlineStr"/>
+      <c r="M56" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=37/2015/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N56" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4513,7 @@
       </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 37/2015/NĐ-CP quy định chi tiết về hợp đồng xây dựng</t>
+          <t>Sửa đổi, bổ sung Nghị định số 37/2015/NĐ-CP về hợp đồng xây dựng (Hết hiệu lực 01/07/2026)</t>
         </is>
       </c>
       <c r="F57" s="13" t="inlineStr">
@@ -4325,10 +4551,14 @@
           <t>ALL, HOP_DONG, LICHSU</t>
         </is>
       </c>
-      <c r="M57" s="15" t="inlineStr"/>
+      <c r="M57" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=50/2021/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N57" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4608,7 @@
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
@@ -4391,10 +4621,14 @@
           <t>ALL, HOP_DONG, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M58" s="8" t="inlineStr"/>
+      <c r="M58" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=02/2023/TT-BXD</t>
+        </is>
+      </c>
       <c r="N58" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4457,10 +4691,14 @@
           <t>THI_NGHIEM_COC, TV-07, XD-01</t>
         </is>
       </c>
-      <c r="M59" s="15" t="inlineStr"/>
+      <c r="M59" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=TCVN%209393%3A2012</t>
+        </is>
+      </c>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4510,7 +4748,7 @@
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
@@ -4523,10 +4761,14 @@
           <t>KHAO_SAT, TV-02</t>
         </is>
       </c>
-      <c r="M60" s="8" t="inlineStr"/>
+      <c r="M60" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=TCVN%209363%3A2012</t>
+        </is>
+      </c>
       <c r="N60" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4818,7 @@
       </c>
       <c r="J61" s="10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K61" s="10" t="inlineStr">
@@ -4589,10 +4831,14 @@
           <t>DO_DAC, TV-01</t>
         </is>
       </c>
-      <c r="M61" s="15" t="inlineStr"/>
+      <c r="M61" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=TCVN%209401%3A2012</t>
+        </is>
+      </c>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4655,10 +4901,14 @@
           <t>BAO_HIEM, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M62" s="8" t="inlineStr"/>
+      <c r="M62" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=08/2022/QH15</t>
+        </is>
+      </c>
       <c r="N62" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4933,7 @@
       </c>
       <c r="E63" s="10" t="inlineStr">
         <is>
-          <t>Quy định về bảo hiểm bắt buộc trách nhiệm dân sự của chủ xe cơ giới, bảo hiểm cháy, nổ bắt buộc, bảo hiểm bắt buộc trong hoạt động đầu tư xây dựng</t>
+          <t>Quy định về bảo hiểm bắt buộc trong hoạt động đầu tư xây dựng</t>
         </is>
       </c>
       <c r="F63" s="13" t="inlineStr">
@@ -4721,10 +4971,14 @@
           <t>BAO_HIEM, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M63" s="15" t="inlineStr"/>
+      <c r="M63" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=67/2023/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N63" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4774,7 +5028,7 @@
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
@@ -4787,10 +5041,14 @@
           <t>KIEM_TOAN, TV-09</t>
         </is>
       </c>
-      <c r="M64" s="8" t="inlineStr"/>
+      <c r="M64" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=67/2011/QH12</t>
+        </is>
+      </c>
       <c r="N64" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4815,7 +5073,7 @@
       </c>
       <c r="E65" s="10" t="inlineStr">
         <is>
-          <t>Ban hành Chuẩn mực kiểm toán Việt Nam số 1000 - Kiểm toán báo cáo quyết toán dự án hoàn thành (VSA 1000)</t>
+          <t>Ban hành Chuẩn mực kiểm toán Việt Nam số 1000 - Kiểm toán quyết toán dự án hoàn thành (VSA 1000)</t>
         </is>
       </c>
       <c r="F65" s="13" t="inlineStr">
@@ -4840,7 +5098,7 @@
       </c>
       <c r="J65" s="10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K65" s="10" t="inlineStr">
@@ -4853,10 +5111,14 @@
           <t>KIEM_TOAN, TV-09</t>
         </is>
       </c>
-      <c r="M65" s="15" t="inlineStr"/>
+      <c r="M65" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=67/2015/TT-BTC</t>
+        </is>
+      </c>
       <c r="N65" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4919,10 +5181,14 @@
           <t>ALL, DAU_TU_CONG, CHU_TRUONG, TV-01, TV-02, TV-03, TV-09</t>
         </is>
       </c>
-      <c r="M66" s="8" t="inlineStr"/>
+      <c r="M66" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=58/2024/QH15</t>
+        </is>
+      </c>
       <c r="N66" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -4947,7 +5213,7 @@
       </c>
       <c r="E67" s="10" t="inlineStr">
         <is>
-          <t>Luật Đầu tư công năm 2019</t>
+          <t>Luật Đầu tư công năm 2019 (Đã hết hiệu lực từ 01/01/2025)</t>
         </is>
       </c>
       <c r="F67" s="13" t="inlineStr">
@@ -4985,10 +5251,14 @@
           <t>ALL, DAU_TU_CONG, LICHSU</t>
         </is>
       </c>
-      <c r="M67" s="15" t="inlineStr"/>
+      <c r="M67" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=39/2019/QH14</t>
+        </is>
+      </c>
       <c r="N67" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5308,7 @@
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
@@ -5051,10 +5321,14 @@
           <t>ALL, DAU_TU_CONG, TV-01, TV-02, TV-03</t>
         </is>
       </c>
-      <c r="M68" s="8" t="inlineStr"/>
+      <c r="M68" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=40/2020/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5109,7 +5383,7 @@
       </c>
       <c r="K69" s="10" t="inlineStr">
         <is>
-          <t>Nghị định xương sống hiện hành về thẩm tra, phê duyệt quyết toán vốn đầu tư công dự án hoàn thành</t>
+          <t>Có hiệu lực từ 26/09/2025; rút ngắn thời gian thanh toán KBNN còn 02 ngày làm việc; hạn lập hồ sơ quyết toán A-B không quá 06 tháng nhóm C (TV-09, XD-01)</t>
         </is>
       </c>
       <c r="L69" s="10" t="inlineStr">
@@ -5117,10 +5391,14 @@
           <t>ALL, QUYET_TOAN, TAI_CHINH, TV-09, XD-01</t>
         </is>
       </c>
-      <c r="M69" s="15" t="inlineStr"/>
+      <c r="M69" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=254/2025/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N69" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5145,7 +5423,7 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Quy định về quản lý, thanh toán, quyết toán dự án sử dụng vốn đầu tư công</t>
+          <t>Quy định quản lý, thanh quyết toán vốn đầu tư công (Hết hiệu lực từ 26/09/2025)</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
@@ -5175,7 +5453,7 @@
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Đã bị thay thế phần lớn bởi NĐ 254/2025/NĐ-CP (chỉ còn áp dụng chuyển tiếp cho một số trường hợp cụ thể)</t>
+          <t>Hết hiệu lực từ 26/09/2025; hồ sơ quyết toán đã nộp trước 26/09/2025 tiếp tục thẩm tra theo NĐ 99/2021</t>
         </is>
       </c>
       <c r="L70" s="3" t="inlineStr">
@@ -5183,10 +5461,14 @@
           <t>ALL, QUYET_TOAN, TAI_CHINH, LICHSU</t>
         </is>
       </c>
-      <c r="M70" s="8" t="inlineStr"/>
+      <c r="M70" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=99/2021/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5249,10 +5531,14 @@
           <t>ALL, QUYET_TOAN, TAI_CHINH, TV-09, XD-01</t>
         </is>
       </c>
-      <c r="M71" s="15" t="inlineStr"/>
+      <c r="M71" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=96/2021/TT-BTC</t>
+        </is>
+      </c>
       <c r="N71" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5563,7 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Thông tư số 96/2021/TT-BTC quy định về hệ thống mẫu biểu hồ sơ quyết toán vốn đầu tư công dự án hoàn thành</t>
+          <t>Sửa đổi, bổ sung Thông tư số 96/2021/TT-BTC về mẫu biểu quyết toán vốn đầu tư công</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
@@ -5315,10 +5601,14 @@
           <t>ALL, QUYET_TOAN, TAI_CHINH, TV-09, XD-01</t>
         </is>
       </c>
-      <c r="M72" s="8" t="inlineStr"/>
+      <c r="M72" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=24/2024/TT-BTC</t>
+        </is>
+      </c>
       <c r="N72" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5663,7 @@
       </c>
       <c r="K73" s="10" t="inlineStr">
         <is>
-          <t>Quy định chi tiết thủ tục thẩm duyệt, nghiệm thu PCCC và cứu nạn cứu hộ số hóa mới nhất</t>
+          <t>Có hiệu lực từ 01/07/2025; cắt giảm danh mục thẩm duyệt PCCC; phân cấp Công an huyện/tỉnh; nộp trực tuyến DVC (05-07 ngày làm việc)</t>
         </is>
       </c>
       <c r="L73" s="10" t="inlineStr">
@@ -5381,10 +5671,14 @@
           <t>PCCC, TV-02, TV-03, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M73" s="15" t="inlineStr"/>
+      <c r="M73" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=105/2025/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N73" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5703,7 @@
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Quy định chi tiết một số điều và biện pháp thi hành Luật Phòng cháy và chữa cháy</t>
+          <t>Quy định chi tiết thi hành Luật Phòng cháy và chữa cháy (Hết hiệu lực 01/07/2025)</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
@@ -5447,10 +5741,14 @@
           <t>PCCC, LICHSU</t>
         </is>
       </c>
-      <c r="M74" s="8" t="inlineStr"/>
+      <c r="M74" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=136/2020/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N74" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5773,7 @@
       </c>
       <c r="E75" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 136/2020/NĐ-CP và Nghị định số 83/2017/NĐ-CP</t>
+          <t>Sửa đổi, bổ sung Nghị định số 136/2020/NĐ-CP về PCCC (Hết hiệu lực 01/07/2025)</t>
         </is>
       </c>
       <c r="F75" s="13" t="inlineStr">
@@ -5513,10 +5811,14 @@
           <t>PCCC, LICHSU</t>
         </is>
       </c>
-      <c r="M75" s="15" t="inlineStr"/>
+      <c r="M75" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=50/2024/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N75" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5579,10 +5881,14 @@
           <t>PCCC, TV-02, TV-03, TV-04, TV-05, XD-01</t>
         </is>
       </c>
-      <c r="M76" s="8" t="inlineStr"/>
+      <c r="M76" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=QCVN%2006%3A2022/BXD</t>
+        </is>
+      </c>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5943,7 @@
       </c>
       <c r="K77" s="10" t="inlineStr">
         <is>
-          <t>Luật nền tảng về Đánh giá tác động môi trường (ĐTM), Giấy phép môi trường và Đăng ký môi trường</t>
+          <t>Luật nền tảng về ĐTM, Giấy phép môi trường và Đăng ký môi trường dự án</t>
         </is>
       </c>
       <c r="L77" s="10" t="inlineStr">
@@ -5645,10 +5951,14 @@
           <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M77" s="15" t="inlineStr"/>
+      <c r="M77" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=72/2020/QH14</t>
+        </is>
+      </c>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5711,10 +6021,14 @@
           <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M78" s="8" t="inlineStr"/>
+      <c r="M78" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=08/2022/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N78" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5739,7 +6053,7 @@
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP quy định chi tiết một số điều của Luật Bảo vệ môi trường</t>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP về bảo vệ môi trường</t>
         </is>
       </c>
       <c r="F79" s="13" t="inlineStr">
@@ -5777,10 +6091,14 @@
           <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M79" s="15" t="inlineStr"/>
+      <c r="M79" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=05/2025/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5805,7 +6123,7 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của các Nghị định quy định chi tiết Luật Bảo vệ môi trường</t>
+          <t>Sửa đổi, bổ sung các Nghị định quy định chi tiết Luật Bảo vệ môi trường</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
@@ -5835,7 +6153,7 @@
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Bãi bỏ cấp đổi GPMT, cho phép lập ĐTM cuốn chiếu theo từng giai đoạn dự án</t>
+          <t>Có hiệu lực từ 29/01/2026; bãi bỏ cấp đổi GPMT phức tạp; phân cấp thẩm định ĐTM; cho phép làm thủ tục môi trường song song với thiết kế xây dựng</t>
         </is>
       </c>
       <c r="L80" s="3" t="inlineStr">
@@ -5843,10 +6161,14 @@
           <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M80" s="8" t="inlineStr"/>
+      <c r="M80" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=48/2026/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N80" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5871,7 +6193,7 @@
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>Nghị quyết về việc tháo gỡ khó khăn, vướng mắc trong thực hiện thủ tục môi trường cho các dự án đầu tư công</t>
+          <t>Nghị quyết tháo gỡ khó khăn trong thực hiện thủ tục môi trường cho dự án đầu tư công</t>
         </is>
       </c>
       <c r="F81" s="13" t="inlineStr">
@@ -5896,7 +6218,7 @@
       </c>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K81" s="10" t="inlineStr">
@@ -5909,10 +6231,14 @@
           <t>MOI_TRUONG, TV-01, TV-02, TV-03, TV-04, XD-01</t>
         </is>
       </c>
-      <c r="M81" s="15" t="inlineStr"/>
+      <c r="M81" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=66.19/2026/NQ-CP</t>
+        </is>
+      </c>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -5975,10 +6301,14 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M82" s="8" t="inlineStr"/>
+      <c r="M82" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=15/2017/QH14</t>
+        </is>
+      </c>
       <c r="N82" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6041,10 +6371,14 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M83" s="15" t="inlineStr"/>
+      <c r="M83" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=151/2017/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6069,7 +6403,7 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 151/2017/NĐ-CP quy định chi tiết một số điều của Luật Quản lý, sử dụng tài sản công</t>
+          <t>Sửa đổi, bổ sung một số điều của Nghị định 151/2017/NĐ-CP về quản lý tài sản công</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
@@ -6107,10 +6441,14 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M84" s="8" t="inlineStr"/>
+      <c r="M84" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=114/2024/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N84" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6473,7 @@
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 151/2017/NĐ-CP về quản lý, sử dụng tài sản công</t>
+          <t>Sửa đổi, bổ sung Nghị định số 151/2017/NĐ-CP về quản lý, sử dụng tài sản công</t>
         </is>
       </c>
       <c r="F85" s="13" t="inlineStr">
@@ -6173,10 +6511,14 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M85" s="15" t="inlineStr"/>
+      <c r="M85" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=186/2025/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6543,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Quy định việc sử dụng kinh phí chi thường xuyên ngân sách nhà nước để thực hiện mua sắm tài sản, trang thiết bị; cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình trong các dự án đã đầu tư xây dựng</t>
+          <t>Quy định việc sử dụng kinh phí chi thường xuyên NSNN để mua sắm, cải tạo, sửa chữa tài sản công</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
@@ -6231,7 +6573,7 @@
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Phân cấp thẩm quyền quyết định dự toán mua sắm, cải tạo tài sản cho Thủ trưởng đơn vị dự toán</t>
+          <t>Có hiệu lực từ 01/05/2026; phân cấp Thủ trưởng đơn vị dự toán BQP phê duyệt dự toán sửa chữa cơ sở vật chất, doanh trại dưới 15 tỷ đồng</t>
         </is>
       </c>
       <c r="L86" s="3" t="inlineStr">
@@ -6239,10 +6581,14 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M86" s="8" t="inlineStr"/>
+      <c r="M86" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=104/2026/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N86" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6613,7 @@
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>Quy định việc sử dụng kinh phí chi thường xuyên ngân sách nhà nước để thực hiện mua sắm tài sản, trang thiết bị; cải tạo, nâng cấp, mở rộng, xây dựng mới hạng mục công trình trong các dự án đã đầu tư xây dựng</t>
+          <t>Quy định sử dụng kinh phí chi thường xuyên mua sắm, cải tạo tài sản công (Hết hiệu lực)</t>
         </is>
       </c>
       <c r="F87" s="13" t="inlineStr">
@@ -6305,10 +6651,14 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, LICHSU</t>
         </is>
       </c>
-      <c r="M87" s="15" t="inlineStr"/>
+      <c r="M87" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=138/2024/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N87" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6683,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Sửa đổi, bổ sung một số điều của Nghị định số 138/2024/NĐ-CP về sử dụng kinh phí chi thường xuyên ngân sách nhà nước</t>
+          <t>Sửa đổi Nghị định 138/2024/NĐ-CP về sử dụng kinh phí chi thường xuyên (Hết hiệu lực)</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
@@ -6371,10 +6721,14 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, LICHSU</t>
         </is>
       </c>
-      <c r="M88" s="8" t="inlineStr"/>
+      <c r="M88" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=98/2025/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N88" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6437,10 +6791,14 @@
           <t>CHI_THUONG_XUYEN, TAI_SAN_CONG, SUA_CHUA, TV-01, TV-02, XD-01</t>
         </is>
       </c>
-      <c r="M89" s="15" t="inlineStr"/>
+      <c r="M89" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=65/2021/TT-BTC</t>
+        </is>
+      </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6503,10 +6861,14 @@
           <t>ALL, THE_THUC, TV-01, TV-02, TV-03, TV-04, TV-05, TV-06, TV-07, TV-08, TV-09, PTV-01, XD-01</t>
         </is>
       </c>
-      <c r="M90" s="8" t="inlineStr"/>
+      <c r="M90" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=30/2020/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N90" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6918,7 @@
       </c>
       <c r="J91" s="10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K91" s="10" t="inlineStr">
@@ -6569,10 +6931,14 @@
           <t>PPP, DAU_TU_CONG</t>
         </is>
       </c>
-      <c r="M91" s="15" t="inlineStr"/>
+      <c r="M91" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=64/2020/QH14</t>
+        </is>
+      </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6988,7 @@
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
@@ -6635,10 +7001,14 @@
           <t>PPP, DAU_TU_CONG</t>
         </is>
       </c>
-      <c r="M92" s="8" t="inlineStr"/>
+      <c r="M92" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=35/2021/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N92" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6701,10 +7071,14 @@
           <t>DAU_TU_KINH_DOANH</t>
         </is>
       </c>
-      <c r="M93" s="15" t="inlineStr"/>
+      <c r="M93" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=61/2020/QH14</t>
+        </is>
+      </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6754,7 +7128,7 @@
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
@@ -6767,10 +7141,14 @@
           <t>DAU_TU_KINH_DOANH</t>
         </is>
       </c>
-      <c r="M94" s="8" t="inlineStr"/>
+      <c r="M94" s="8" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=31/2021/N%C4%90-CP</t>
+        </is>
+      </c>
       <c r="N94" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>
@@ -6820,7 +7198,7 @@
       </c>
       <c r="J95" s="10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Văn bản gốc / Ban hành lần đầu</t>
         </is>
       </c>
       <c r="K95" s="10" t="inlineStr">
@@ -6833,10 +7211,14 @@
           <t>ALL, BQP, PHAN_CAP, QLDA, TV-01, TV-02, TV-03, TV-04, TV-05, TV-08, XD-01</t>
         </is>
       </c>
-      <c r="M95" s="15" t="inlineStr"/>
+      <c r="M95" s="15" t="inlineStr">
+        <is>
+          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=15/VBHN-BQP</t>
+        </is>
+      </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>2026-08-21 17:02</t>
+          <t>2026-08-22 07:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Chuyen link tra cuu sang Google Search tranh loi 404 PageNotFound cua TVPL
</commit_message>
<xml_diff>
--- a/Kho_Can_Cu_Phap_Ly.xlsx
+++ b/Kho_Can_Cu_Phap_Ly.xlsx
@@ -703,12 +703,12 @@
       </c>
       <c r="M2" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=47/2024/QH15</t>
+          <t>https://www.google.com/search?q=47/2024/QH15%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -773,12 +773,12 @@
       </c>
       <c r="M3" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=30/2009/QH12</t>
+          <t>https://www.google.com/search?q=30/2009/QH12%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N3" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -843,12 +843,12 @@
       </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=178/2025/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=178/2025/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="M5" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=44/2015/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=44/2015/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="M6" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=04/2022/TT-BXD</t>
+          <t>https://www.google.com/search?q=04/2022/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1053,12 +1053,12 @@
       </c>
       <c r="M7" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=20/2019/TT-BXD</t>
+          <t>https://www.google.com/search?q=20/2019/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N7" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1123,12 +1123,12 @@
       </c>
       <c r="M8" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=QCVN%2001%3A2021/BXD</t>
+          <t>https://www.google.com/search?q=QCVN%2001%3A2021/BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1193,12 +1193,12 @@
       </c>
       <c r="M9" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=27/2018/QH14</t>
+          <t>https://www.google.com/search?q=27/2018/QH14%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N9" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1263,12 +1263,12 @@
       </c>
       <c r="M10" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=27/2019/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=27/2019/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1333,12 @@
       </c>
       <c r="M11" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=135/2025/QH15</t>
+          <t>https://www.google.com/search?q=135/2025/QH15%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="M12" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=50/2014/QH13</t>
+          <t>https://www.google.com/search?q=50/2014/QH13%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1473,12 +1473,12 @@
       </c>
       <c r="M13" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=62/2020/QH14</t>
+          <t>https://www.google.com/search?q=62/2020/QH14%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1543,12 +1543,12 @@
       </c>
       <c r="M14" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=217/2026/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=217/2026/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1613,12 +1613,12 @@
       </c>
       <c r="M15" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=175/2024/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=175/2024/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1683,12 +1683,12 @@
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=15/2021/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=15/2021/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="M17" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=35/2023/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=35/2023/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1823,12 +1823,12 @@
       </c>
       <c r="M18" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=84/2015/QH13</t>
+          <t>https://www.google.com/search?q=84/2015/QH13%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1893,12 +1893,12 @@
       </c>
       <c r="M19" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=22/2023/QH15</t>
+          <t>https://www.google.com/search?q=22/2023/QH15%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -1963,12 +1963,12 @@
       </c>
       <c r="M20" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=57/2024/QH15</t>
+          <t>https://www.google.com/search?q=57/2024/QH15%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2033,12 +2033,12 @@
       </c>
       <c r="M21" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=90/2025/QH15</t>
+          <t>https://www.google.com/search?q=90/2025/QH15%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2103,12 +2103,12 @@
       </c>
       <c r="M22" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=43/2013/QH13</t>
+          <t>https://www.google.com/search?q=43/2013/QH13%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2173,12 +2173,12 @@
       </c>
       <c r="M23" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=214/2025/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=214/2025/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N23" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2243,12 +2243,12 @@
       </c>
       <c r="M24" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=24/2024/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=24/2024/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>Bị thay thế bởi 24/2024/NĐ-CP</t>
+          <t>Bị thay thế bởi Nghị định 24/2024/NĐ-CP, Bị thay thế bởi 24/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="K25" s="10" t="inlineStr">
@@ -2313,12 +2313,12 @@
       </c>
       <c r="M25" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=63/2014/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=63/2014/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N25" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2383,12 +2383,12 @@
       </c>
       <c r="M26" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=79/2025/TT-BTC</t>
+          <t>https://www.google.com/search?q=79/2025/TT-BTC%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2453,12 +2453,12 @@
       </c>
       <c r="M27" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=06/2024/TT-BKH%C4%90T</t>
+          <t>https://www.google.com/search?q=06/2024/TT-BKH%C4%90T%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N27" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2523,12 +2523,12 @@
       </c>
       <c r="M28" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=80/2025/TT-BTC</t>
+          <t>https://www.google.com/search?q=80/2025/TT-BTC%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2593,12 +2593,12 @@
       </c>
       <c r="M29" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=206/2026/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=206/2026/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N29" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2663,12 +2663,12 @@
       </c>
       <c r="M30" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=10/2021/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=10/2021/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2733,12 +2733,12 @@
       </c>
       <c r="M31" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=36/2026/TT-BXD</t>
+          <t>https://www.google.com/search?q=36/2026/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N31" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2803,12 +2803,12 @@
       </c>
       <c r="M32" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=38/2026/TT-BXD</t>
+          <t>https://www.google.com/search?q=38/2026/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2873,12 +2873,12 @@
       </c>
       <c r="M33" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=12/2021/TT-BXD</t>
+          <t>https://www.google.com/search?q=12/2021/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N33" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -2943,12 +2943,12 @@
       </c>
       <c r="M34" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=09/2024/TT-BXD</t>
+          <t>https://www.google.com/search?q=09/2024/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3013,12 +3013,12 @@
       </c>
       <c r="M35" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=01/2025/TT-BXD</t>
+          <t>https://www.google.com/search?q=01/2025/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N35" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="M36" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=11/2021/TT-BXD</t>
+          <t>https://www.google.com/search?q=11/2021/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3153,12 +3153,12 @@
       </c>
       <c r="M37" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=14/2023/TT-BXD</t>
+          <t>https://www.google.com/search?q=14/2023/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N37" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3223,12 +3223,12 @@
       </c>
       <c r="M38" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=13/2021/TT-BXD</t>
+          <t>https://www.google.com/search?q=13/2021/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3293,12 +3293,12 @@
       </c>
       <c r="M39" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=425/Q%C4%90-BXD</t>
+          <t>https://www.google.com/search?q=425/Q%C4%90-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N39" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3363,12 +3363,12 @@
       </c>
       <c r="M40" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=510/Q%C4%90-BXD</t>
+          <t>https://www.google.com/search?q=510/Q%C4%90-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3433,12 +3433,12 @@
       </c>
       <c r="M41" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=101/2026/TT-BQP</t>
+          <t>https://www.google.com/search?q=101/2026/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N41" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3503,12 +3503,12 @@
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=102/2026/TT-BQP</t>
+          <t>https://www.google.com/search?q=102/2026/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3573,12 +3573,12 @@
       </c>
       <c r="M43" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=128/2021/TT-BQP</t>
+          <t>https://www.google.com/search?q=128/2021/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N43" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3643,12 +3643,12 @@
       </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=73/2023/TT-BQP</t>
+          <t>https://www.google.com/search?q=73/2023/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N44" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3713,12 +3713,12 @@
       </c>
       <c r="M45" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=120/2024/TT-BQP</t>
+          <t>https://www.google.com/search?q=120/2024/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N45" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3783,12 +3783,12 @@
       </c>
       <c r="M46" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=174/2021/TT-BQP</t>
+          <t>https://www.google.com/search?q=174/2021/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3853,12 +3853,12 @@
       </c>
       <c r="M47" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=24/2025/TT-BQP</t>
+          <t>https://www.google.com/search?q=24/2025/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N47" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3923,12 +3923,12 @@
       </c>
       <c r="M48" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=36/2023/TT-BQP</t>
+          <t>https://www.google.com/search?q=36/2023/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N48" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -3993,12 +3993,12 @@
       </c>
       <c r="M49" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=150/2018/TT-BQP</t>
+          <t>https://www.google.com/search?q=150/2018/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N49" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4063,12 +4063,12 @@
       </c>
       <c r="M50" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=94/2024/TT-BQP</t>
+          <t>https://www.google.com/search?q=94/2024/TT-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N50" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4133,12 +4133,12 @@
       </c>
       <c r="M51" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=35/Q%C4%90-TTg</t>
+          <t>https://www.google.com/search?q=35/Q%C4%90-TTg%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N51" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4203,12 +4203,12 @@
       </c>
       <c r="M52" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=207/2026/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=207/2026/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4273,12 +4273,12 @@
       </c>
       <c r="M53" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=06/2021/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=06/2021/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N53" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4343,12 +4343,12 @@
       </c>
       <c r="M54" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=10/2021/TT-BXD</t>
+          <t>https://www.google.com/search?q=10/2021/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4413,12 +4413,12 @@
       </c>
       <c r="M55" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=210/2026/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=210/2026/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N55" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4483,12 +4483,12 @@
       </c>
       <c r="M56" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=37/2015/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=37/2015/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4553,12 +4553,12 @@
       </c>
       <c r="M57" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=50/2021/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=50/2021/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N57" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4623,12 +4623,12 @@
       </c>
       <c r="M58" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=02/2023/TT-BXD</t>
+          <t>https://www.google.com/search?q=02/2023/TT-BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N58" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4693,12 +4693,12 @@
       </c>
       <c r="M59" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=TCVN%209393%3A2012</t>
+          <t>https://www.google.com/search?q=TCVN%209393%3A2012%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4763,12 +4763,12 @@
       </c>
       <c r="M60" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=TCVN%209363%3A2012</t>
+          <t>https://www.google.com/search?q=TCVN%209363%3A2012%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N60" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4833,12 +4833,12 @@
       </c>
       <c r="M61" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=TCVN%209401%3A2012</t>
+          <t>https://www.google.com/search?q=TCVN%209401%3A2012%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4903,12 +4903,12 @@
       </c>
       <c r="M62" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=08/2022/QH15</t>
+          <t>https://www.google.com/search?q=08/2022/QH15%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N62" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -4973,12 +4973,12 @@
       </c>
       <c r="M63" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=67/2023/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=67/2023/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N63" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5043,12 +5043,12 @@
       </c>
       <c r="M64" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=67/2011/QH12</t>
+          <t>https://www.google.com/search?q=67/2011/QH12%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N64" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5113,12 +5113,12 @@
       </c>
       <c r="M65" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=67/2015/TT-BTC</t>
+          <t>https://www.google.com/search?q=67/2015/TT-BTC%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N65" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5183,12 +5183,12 @@
       </c>
       <c r="M66" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=58/2024/QH15</t>
+          <t>https://www.google.com/search?q=58/2024/QH15%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N66" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5253,12 +5253,12 @@
       </c>
       <c r="M67" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=39/2019/QH14</t>
+          <t>https://www.google.com/search?q=39/2019/QH14%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N67" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5323,12 +5323,12 @@
       </c>
       <c r="M68" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=40/2020/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=40/2020/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5393,12 +5393,12 @@
       </c>
       <c r="M69" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=254/2025/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=254/2025/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N69" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5463,12 +5463,12 @@
       </c>
       <c r="M70" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=99/2021/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=99/2021/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5533,12 +5533,12 @@
       </c>
       <c r="M71" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=96/2021/TT-BTC</t>
+          <t>https://www.google.com/search?q=96/2021/TT-BTC%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N71" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5603,12 +5603,12 @@
       </c>
       <c r="M72" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=24/2024/TT-BTC</t>
+          <t>https://www.google.com/search?q=24/2024/TT-BTC%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N72" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5673,12 +5673,12 @@
       </c>
       <c r="M73" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=105/2025/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=105/2025/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N73" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5743,12 +5743,12 @@
       </c>
       <c r="M74" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=136/2020/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=136/2020/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N74" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5813,12 +5813,12 @@
       </c>
       <c r="M75" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=50/2024/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=50/2024/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N75" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5883,12 +5883,12 @@
       </c>
       <c r="M76" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=QCVN%2006%3A2022/BXD</t>
+          <t>https://www.google.com/search?q=QCVN%2006%3A2022/BXD%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -5953,12 +5953,12 @@
       </c>
       <c r="M77" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=72/2020/QH14</t>
+          <t>https://www.google.com/search?q=72/2020/QH14%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6023,12 +6023,12 @@
       </c>
       <c r="M78" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=08/2022/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=08/2022/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N78" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6093,12 +6093,12 @@
       </c>
       <c r="M79" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=05/2025/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=05/2025/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6163,12 +6163,12 @@
       </c>
       <c r="M80" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=48/2026/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=48/2026/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N80" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6233,12 +6233,12 @@
       </c>
       <c r="M81" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=66.19/2026/NQ-CP</t>
+          <t>https://www.google.com/search?q=19/2026/NQ-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6303,12 +6303,12 @@
       </c>
       <c r="M82" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=15/2017/QH14</t>
+          <t>https://www.google.com/search?q=15/2017/QH14%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N82" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6373,12 +6373,12 @@
       </c>
       <c r="M83" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=151/2017/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=151/2017/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6443,12 +6443,12 @@
       </c>
       <c r="M84" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=114/2024/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=114/2024/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N84" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6513,12 +6513,12 @@
       </c>
       <c r="M85" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=186/2025/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=186/2025/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6583,12 +6583,12 @@
       </c>
       <c r="M86" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=104/2026/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=104/2026/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N86" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6653,12 +6653,12 @@
       </c>
       <c r="M87" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=138/2024/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=138/2024/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N87" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6723,12 +6723,12 @@
       </c>
       <c r="M88" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=98/2025/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=98/2025/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N88" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6793,12 +6793,12 @@
       </c>
       <c r="M89" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=65/2021/TT-BTC</t>
+          <t>https://www.google.com/search?q=65/2021/TT-BTC%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6863,12 +6863,12 @@
       </c>
       <c r="M90" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=30/2020/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=30/2020/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N90" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -6933,12 +6933,12 @@
       </c>
       <c r="M91" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=64/2020/QH14</t>
+          <t>https://www.google.com/search?q=64/2020/QH14%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -7003,12 +7003,12 @@
       </c>
       <c r="M92" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=35/2021/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=35/2021/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N92" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -7073,12 +7073,12 @@
       </c>
       <c r="M93" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=61/2020/QH14</t>
+          <t>https://www.google.com/search?q=61/2020/QH14%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -7143,12 +7143,12 @@
       </c>
       <c r="M94" s="8" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=31/2021/N%C4%90-CP</t>
+          <t>https://www.google.com/search?q=31/2021/N%C4%90-CP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N94" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>
@@ -7213,12 +7213,12 @@
       </c>
       <c r="M95" s="15" t="inlineStr">
         <is>
-          <t>https://thuvienphapluat.vn/page/tim-van-ban.aspx?keyword=15/VBHN-BQP</t>
+          <t>https://www.google.com/search?q=15/VBHN-BQP%20thuvienphapluat</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>2026-08-22 07:11</t>
+          <t>2026-08-22 07:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Cai tien _fallback_local_analysis doc du lieu dong va tra cuu CSDL 94 van ban
</commit_message>
<xml_diff>
--- a/Kho_Can_Cu_Phap_Ly.xlsx
+++ b/Kho_Can_Cu_Phap_Ly.xlsx
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N95"/>
+  <dimension ref="A1:N96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2151,14 +2151,14 @@
           <t>04/08/2025</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>Đang có hiệu lực</t>
+      <c r="I23" s="14" t="inlineStr">
+        <is>
+          <t>Hết hiệu lực</t>
         </is>
       </c>
       <c r="J23" s="10" t="inlineStr">
         <is>
-          <t>Thay thế Nghị định 24/2024/NĐ-CP và Nghị định 63/2014/NĐ-CP</t>
+          <t>Thay thế Nghị định 24/2024/NĐ-CP và Nghị định 63/2014/NĐ-CP, Bị thay thế bởi 24/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="K23" s="10" t="inlineStr">
@@ -7219,6 +7219,76 @@
       <c r="N95" s="11" t="inlineStr">
         <is>
           <t>2026-08-22 07:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="26" customHeight="1">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; Đấu thầu</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Nghị định</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>42/2026/QĐ-TTg</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Quyết định 42/2026/QĐ-TTg Ban hành Danh mục lĩnh vực, cơ sở phát thải khí nhà kính phải thực hiện kiểm kê khí nhà kính (cập nhật)</t>
+        </is>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>Thủ tướng Chính phủ</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="I96" s="7" t="inlineStr">
+        <is>
+          <t>Đang có hiệu lực</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>Áp dụng theo quy định ban hành mới</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>Quyết định 42/2026/QĐ-TTg Ban hành Danh mục lĩnh vực, cơ sở phát thải khí nhà kính phải thực hiện kiểm kê khí nhà kính (cập nhật) Quy định danh mục các lĩnh vực sản xuất, công trìn</t>
+        </is>
+      </c>
+      <c r="L96" s="3" t="inlineStr">
+        <is>
+          <t>#Xây_dựng, #Đấu_thầu, #Dự_án</t>
+        </is>
+      </c>
+      <c r="M96" s="8" t="inlineStr">
+        <is>
+          <t>https://telegra.ph/BÁO-CÁO-PHÂN-TÍCH-Quyết-định-422026QĐ-TTg-Ban-hành-Danh-mục-lĩnh-vực-cơ-sở-phát-thải-khí-nhà-kín-08-22</t>
+        </is>
+      </c>
+      <c r="N96" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-22 07:46</t>
         </is>
       </c>
     </row>

</xml_diff>